<commit_message>
Implement double-column sidebar, dark/light theme toggle, centralized calculations, and fix tablet sidebar layout
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1197,22 +1197,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>30/04/2026</v>
+        <v>01/01/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>Apr26</v>
+        <v>May26</v>
       </c>
       <c r="C4" t="str">
         <v>OPEX</v>
       </c>
       <c r="D4" t="str">
-        <v>Salary</v>
+        <v>Fixed Costs</v>
       </c>
       <c r="E4" t="str">
-        <v>Employee 3</v>
+        <v>ค่าเช่าร้าน 2 เดือนพฤษภาคม</v>
       </c>
       <c r="F4">
-        <v>12000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="5">
@@ -1229,10 +1229,10 @@
         <v>Salary</v>
       </c>
       <c r="E5" t="str">
-        <v>Employee 4</v>
+        <v>Employee 3</v>
       </c>
       <c r="F5">
-        <v>6000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="6">
@@ -1246,13 +1246,13 @@
         <v>OPEX</v>
       </c>
       <c r="D6" t="str">
-        <v>Fixed Costs</v>
+        <v>Salary</v>
       </c>
       <c r="E6" t="str">
-        <v>Rent</v>
+        <v>Employee 4</v>
       </c>
       <c r="F6">
-        <v>30000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="7">
@@ -1266,18 +1266,98 @@
         <v>OPEX</v>
       </c>
       <c r="D7" t="str">
+        <v>Fixed Costs</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="F7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>30/04/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Apr26</v>
+      </c>
+      <c r="C8" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D8" t="str">
         <v>Investment</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E8" t="str">
         <v>Stock (Allocated 17.1%)</v>
       </c>
-      <c r="F7">
+      <c r="F8">
         <v>2052</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>31/05/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C9" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Employee 3</v>
+      </c>
+      <c r="F9">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>31/05/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C10" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Employee 4</v>
+      </c>
+      <c r="F10">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>31/05/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C11" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Stock (Allocated 40.25%)</v>
+      </c>
+      <c r="F11">
+        <v>4830</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2832,7 +2912,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2954,16 +3034,16 @@
         <v>4100</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L3">
         <v>31</v>
@@ -2972,7 +3052,7 @@
         <v>12</v>
       </c>
       <c r="N3">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="O3">
         <v>11</v>
@@ -2990,13 +3070,13 @@
         <v>0</v>
       </c>
       <c r="T3">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="U3">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="V3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W3">
         <v>2</v>
@@ -3011,16 +3091,16 @@
         <v>1.5</v>
       </c>
       <c r="AA3">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="AB3">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="AC3">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="AD3">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3218,16 +3298,16 @@
         <v>6570</v>
       </c>
       <c r="D6">
-        <v>5070</v>
+        <v>4950</v>
       </c>
       <c r="E6">
         <v>120</v>
       </c>
       <c r="F6">
-        <v>4950</v>
+        <v>4830</v>
       </c>
       <c r="G6">
-        <v>1500</v>
+        <v>1620</v>
       </c>
       <c r="H6">
         <v>23</v>
@@ -3236,7 +3316,7 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -3257,7 +3337,7 @@
         <v>9</v>
       </c>
       <c r="Q6">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -3310,28 +3390,28 @@
         <v>5550</v>
       </c>
       <c r="D7">
-        <v>3680</v>
+        <v>3560</v>
       </c>
       <c r="E7">
         <v>120</v>
       </c>
       <c r="F7">
-        <v>3560</v>
+        <v>3440</v>
       </c>
       <c r="G7">
         <v>1990</v>
       </c>
       <c r="H7">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="K7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L7">
         <v>12</v>
@@ -3349,7 +3429,7 @@
         <v>6</v>
       </c>
       <c r="Q7">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -3358,13 +3438,13 @@
         <v>0</v>
       </c>
       <c r="T7">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="U7">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="V7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W7">
         <v>1</v>
@@ -3379,13 +3459,13 @@
         <v>1</v>
       </c>
       <c r="AA7">
+        <v>6</v>
+      </c>
+      <c r="AB7">
+        <v>26</v>
+      </c>
+      <c r="AC7">
         <v>3</v>
-      </c>
-      <c r="AB7">
-        <v>13</v>
-      </c>
-      <c r="AC7">
-        <v>6</v>
       </c>
       <c r="AD7">
         <v>0</v>
@@ -3399,7 +3479,7 @@
         <v>Wed</v>
       </c>
       <c r="C8">
-        <v>4830</v>
+        <v>4710</v>
       </c>
       <c r="D8">
         <v>3890</v>
@@ -3411,34 +3491,34 @@
         <v>3770</v>
       </c>
       <c r="G8">
-        <v>940</v>
+        <v>820</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N8">
         <v>0</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q8">
         <v>81</v>
@@ -3450,13 +3530,13 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>11.5</v>
+        <v>0.5</v>
       </c>
       <c r="U8">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="V8">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="W8">
         <v>1</v>
@@ -3471,16 +3551,16 @@
         <v>1</v>
       </c>
       <c r="AA8">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="AB8">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="AC8">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="AD8">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3491,7 +3571,7 @@
         <v>Thu</v>
       </c>
       <c r="C9">
-        <v>3080</v>
+        <v>3020</v>
       </c>
       <c r="D9">
         <v>2160</v>
@@ -3503,7 +3583,7 @@
         <v>2100</v>
       </c>
       <c r="G9">
-        <v>920</v>
+        <v>860</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -3598,7 +3678,7 @@
         <v>1440</v>
       </c>
       <c r="H10">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -3625,7 +3705,7 @@
         <v>10</v>
       </c>
       <c r="Q10">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="R10">
         <v>0</v>
@@ -3681,43 +3761,43 @@
         <v>3601</v>
       </c>
       <c r="E11">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>3481</v>
+        <v>3601</v>
       </c>
       <c r="G11">
         <v>2160</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L11">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N11">
         <v>0</v>
       </c>
       <c r="O11">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="P11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q11">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -3732,7 +3812,7 @@
         <v>35</v>
       </c>
       <c r="V11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W11">
         <v>1</v>
@@ -3747,13 +3827,13 @@
         <v>1</v>
       </c>
       <c r="AA11">
+        <v>8</v>
+      </c>
+      <c r="AB11">
+        <v>9</v>
+      </c>
+      <c r="AC11">
         <v>4</v>
-      </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-      <c r="AC11">
-        <v>9</v>
       </c>
       <c r="AD11">
         <v>0</v>
@@ -3782,34 +3862,34 @@
         <v>1440</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="M12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q12">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -3951,7 +4031,7 @@
         <v>Tue</v>
       </c>
       <c r="C14">
-        <v>3520</v>
+        <v>3400</v>
       </c>
       <c r="D14">
         <v>2550</v>
@@ -3963,10 +4043,10 @@
         <v>2430</v>
       </c>
       <c r="G14">
-        <v>970</v>
+        <v>850</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -3975,13 +4055,13 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="L14">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M14">
-        <v>13.5</v>
+        <v>10</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -3990,10 +4070,10 @@
         <v>8</v>
       </c>
       <c r="P14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q14">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="R14">
         <v>0</v>
@@ -4005,7 +4085,7 @@
         <v>4</v>
       </c>
       <c r="U14">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="V14">
         <v>1</v>
@@ -4023,13 +4103,13 @@
         <v>1</v>
       </c>
       <c r="AA14">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AB14">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AC14">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AD14">
         <v>0</v>
@@ -4058,31 +4138,31 @@
         <v>2190</v>
       </c>
       <c r="H15">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="J15">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="K15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L15">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M15">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N15">
         <v>0</v>
       </c>
       <c r="O15">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q15">
         <v>98</v>
@@ -4094,37 +4174,37 @@
         <v>0</v>
       </c>
       <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15">
+        <v>9</v>
+      </c>
+      <c r="V15">
+        <v>10</v>
+      </c>
+      <c r="W15">
+        <v>1</v>
+      </c>
+      <c r="X15">
+        <v>1</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15">
+        <v>1</v>
+      </c>
+      <c r="AA15">
+        <v>16</v>
+      </c>
+      <c r="AB15">
         <v>23</v>
       </c>
-      <c r="U15">
-        <v>42</v>
-      </c>
-      <c r="V15">
-        <v>5</v>
-      </c>
-      <c r="W15">
-        <v>1</v>
-      </c>
-      <c r="X15">
-        <v>1</v>
-      </c>
-      <c r="Y15">
-        <v>1</v>
-      </c>
-      <c r="Z15">
-        <v>1</v>
-      </c>
-      <c r="AA15">
-        <v>8</v>
-      </c>
-      <c r="AB15">
-        <v>9</v>
-      </c>
       <c r="AC15">
         <v>0</v>
       </c>
       <c r="AD15">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -4138,16 +4218,16 @@
         <v>5550</v>
       </c>
       <c r="D16">
-        <v>4520</v>
+        <v>4320</v>
       </c>
       <c r="E16">
         <v>120</v>
       </c>
       <c r="F16">
-        <v>4400</v>
+        <v>4200</v>
       </c>
       <c r="G16">
-        <v>1030</v>
+        <v>1230</v>
       </c>
       <c r="H16">
         <v>25</v>
@@ -4186,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="T16">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="U16">
         <v>11</v>
@@ -4219,57 +4299,149 @@
         <v>0</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>15/05/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C17">
+        <v>7180</v>
+      </c>
+      <c r="D17">
+        <v>5830</v>
+      </c>
+      <c r="E17">
+        <v>120</v>
+      </c>
+      <c r="F17">
+        <v>5710</v>
+      </c>
+      <c r="G17">
+        <v>1350</v>
+      </c>
+      <c r="H17">
+        <v>24</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>51</v>
+      </c>
+      <c r="K17">
+        <v>10</v>
+      </c>
+      <c r="L17">
+        <v>11</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>12</v>
+      </c>
+      <c r="P17">
+        <v>12</v>
+      </c>
+      <c r="Q17">
+        <v>124</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>12</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>2</v>
+      </c>
+      <c r="X17">
+        <v>1</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <v>1</v>
+      </c>
+      <c r="AA17">
+        <v>8</v>
+      </c>
+      <c r="AB17">
+        <v>36</v>
+      </c>
+      <c r="AC17">
+        <v>6</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TOTAL</v>
+        <v>16/05/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>14 days</v>
+        <v>Sat</v>
       </c>
       <c r="C18">
-        <v>89111</v>
+        <v>4590</v>
       </c>
       <c r="D18">
-        <v>61841</v>
+        <v>3030</v>
       </c>
       <c r="E18">
-        <v>1710</v>
+        <v>60</v>
       </c>
       <c r="F18">
-        <v>60131</v>
+        <v>2970</v>
       </c>
       <c r="G18">
-        <v>27390</v>
+        <v>1560</v>
       </c>
       <c r="H18">
-        <v>542</v>
+        <v>17</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>304</v>
+        <v>31</v>
       </c>
       <c r="K18">
-        <v>839</v>
+        <v>2</v>
       </c>
       <c r="L18">
-        <v>3212</v>
+        <v>11</v>
       </c>
       <c r="M18">
-        <v>1746</v>
+        <v>6</v>
       </c>
       <c r="N18">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="O18">
-        <v>1972</v>
+        <v>8</v>
       </c>
       <c r="P18">
-        <v>1682</v>
+        <v>6</v>
       </c>
       <c r="Q18">
-        <v>19470</v>
+        <v>82</v>
       </c>
       <c r="R18">
         <v>0</v>
@@ -4278,131 +4450,1511 @@
         <v>0</v>
       </c>
       <c r="T18">
-        <v>142</v>
+        <v>14</v>
       </c>
       <c r="U18">
-        <v>299.5</v>
+        <v>31</v>
       </c>
       <c r="V18">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="W18">
-        <v>20.5</v>
+        <v>0.5</v>
       </c>
       <c r="X18">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="Y18">
-        <v>10.5</v>
+        <v>1</v>
       </c>
       <c r="Z18">
-        <v>18.5</v>
+        <v>1</v>
       </c>
       <c r="AA18">
-        <v>133</v>
+        <v>6</v>
       </c>
       <c r="AB18">
-        <v>169</v>
+        <v>8</v>
       </c>
       <c r="AC18">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="AD18">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>17/05/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C19">
+        <v>3570</v>
+      </c>
+      <c r="D19">
+        <v>2000</v>
+      </c>
+      <c r="E19">
+        <v>120</v>
+      </c>
+      <c r="F19">
+        <v>1880</v>
+      </c>
+      <c r="G19">
+        <v>1570</v>
+      </c>
+      <c r="H19">
+        <v>18</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>29</v>
+      </c>
+      <c r="K19">
+        <v>3</v>
+      </c>
+      <c r="L19">
+        <v>4</v>
+      </c>
+      <c r="M19">
+        <v>2</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19">
+        <v>5</v>
+      </c>
+      <c r="Q19">
+        <v>62</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>18</v>
+      </c>
+      <c r="U19">
+        <v>29</v>
+      </c>
+      <c r="V19">
+        <v>3</v>
+      </c>
+      <c r="W19">
+        <v>1</v>
+      </c>
+      <c r="X19">
+        <v>1</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>2</v>
+      </c>
+      <c r="AB19">
+        <v>0</v>
+      </c>
+      <c r="AC19">
+        <v>5</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>18/05/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C20">
+        <v>6110</v>
+      </c>
+      <c r="D20">
+        <v>4350</v>
+      </c>
+      <c r="E20">
+        <v>120</v>
+      </c>
+      <c r="F20">
+        <v>4230</v>
+      </c>
+      <c r="G20">
+        <v>1760</v>
+      </c>
+      <c r="H20">
+        <v>24</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>44</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>23</v>
+      </c>
+      <c r="M20">
+        <v>6</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>13</v>
+      </c>
+      <c r="Q20">
+        <v>110</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>1</v>
+      </c>
+      <c r="U20">
+        <v>10</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>2</v>
+      </c>
+      <c r="X20">
+        <v>2</v>
+      </c>
+      <c r="Y20">
+        <v>1.5</v>
+      </c>
+      <c r="Z20">
+        <v>1.5</v>
+      </c>
+      <c r="AA20">
+        <v>12</v>
+      </c>
+      <c r="AB20">
+        <v>0</v>
+      </c>
+      <c r="AC20">
+        <v>10</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>19/05/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C21">
+        <v>2830</v>
+      </c>
+      <c r="D21">
+        <v>2380</v>
+      </c>
+      <c r="E21">
+        <v>60</v>
+      </c>
+      <c r="F21">
+        <v>2320</v>
+      </c>
+      <c r="G21">
+        <v>450</v>
+      </c>
+      <c r="H21">
+        <v>15</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>2</v>
+      </c>
+      <c r="L21">
+        <v>9</v>
+      </c>
+      <c r="M21">
+        <v>2</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>3</v>
+      </c>
+      <c r="P21">
+        <v>2</v>
+      </c>
+      <c r="Q21">
+        <v>33</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>9</v>
+      </c>
+      <c r="U21">
+        <v>23</v>
+      </c>
+      <c r="V21">
+        <v>4</v>
+      </c>
+      <c r="W21">
+        <v>1</v>
+      </c>
+      <c r="X21">
+        <v>0.5</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <v>2</v>
+      </c>
+      <c r="AB21">
+        <v>9</v>
+      </c>
+      <c r="AC21">
+        <v>3</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>20/05/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C22">
+        <v>2480</v>
+      </c>
+      <c r="D22">
+        <v>1870</v>
+      </c>
+      <c r="E22">
+        <v>60</v>
+      </c>
+      <c r="F22">
+        <v>1810</v>
+      </c>
+      <c r="G22">
+        <v>610</v>
+      </c>
+      <c r="H22">
+        <v>16</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>16</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>6</v>
+      </c>
+      <c r="M22">
+        <v>2</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22">
+        <v>2</v>
+      </c>
+      <c r="Q22">
+        <v>43</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>0.5</v>
+      </c>
+      <c r="U22">
+        <v>4</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+      <c r="W22">
+        <v>0.5</v>
+      </c>
+      <c r="X22">
+        <v>0.5</v>
+      </c>
+      <c r="Y22">
+        <v>0.5</v>
+      </c>
+      <c r="Z22">
+        <v>0.5</v>
+      </c>
+      <c r="AA22">
+        <v>4</v>
+      </c>
+      <c r="AB22">
+        <v>3</v>
+      </c>
+      <c r="AC22">
+        <v>1</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C23">
+        <v>5660</v>
+      </c>
+      <c r="D23">
+        <v>3940</v>
+      </c>
+      <c r="E23">
+        <v>120</v>
+      </c>
+      <c r="F23">
+        <v>3820</v>
+      </c>
+      <c r="G23">
+        <v>1720</v>
+      </c>
+      <c r="H23">
+        <v>36</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>3</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23">
+        <v>5</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>5</v>
+      </c>
+      <c r="P23">
+        <v>10</v>
+      </c>
+      <c r="Q23">
+        <v>69</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>21</v>
+      </c>
+      <c r="U23">
+        <v>4</v>
+      </c>
+      <c r="V23">
+        <v>4</v>
+      </c>
+      <c r="W23">
+        <v>1</v>
+      </c>
+      <c r="X23">
+        <v>1</v>
+      </c>
+      <c r="Y23">
+        <v>1</v>
+      </c>
+      <c r="Z23">
+        <v>1</v>
+      </c>
+      <c r="AA23">
+        <v>5</v>
+      </c>
+      <c r="AB23">
+        <v>7</v>
+      </c>
+      <c r="AC23">
+        <v>6</v>
+      </c>
+      <c r="AD23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>23/05/2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C24">
+        <v>5740</v>
+      </c>
+      <c r="D24">
+        <v>3260</v>
+      </c>
+      <c r="E24">
+        <v>120</v>
+      </c>
+      <c r="F24">
+        <v>3140</v>
+      </c>
+      <c r="G24">
+        <v>2480</v>
+      </c>
+      <c r="H24">
+        <v>24</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>44</v>
+      </c>
+      <c r="K24">
+        <v>4</v>
+      </c>
+      <c r="L24">
+        <v>11</v>
+      </c>
+      <c r="M24">
+        <v>6</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>7</v>
+      </c>
+      <c r="P24">
+        <v>4</v>
+      </c>
+      <c r="Q24">
+        <v>100</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>1</v>
+      </c>
+      <c r="U24">
+        <v>7</v>
+      </c>
+      <c r="V24">
+        <v>8</v>
+      </c>
+      <c r="W24">
+        <v>1</v>
+      </c>
+      <c r="X24">
+        <v>1</v>
+      </c>
+      <c r="Y24">
+        <v>1</v>
+      </c>
+      <c r="Z24">
+        <v>1</v>
+      </c>
+      <c r="AA24">
+        <v>12</v>
+      </c>
+      <c r="AB24">
+        <v>21</v>
+      </c>
+      <c r="AC24">
+        <v>2</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>24/05/2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C25">
+        <v>5920</v>
+      </c>
+      <c r="D25">
+        <v>4390</v>
+      </c>
+      <c r="E25">
+        <v>120</v>
+      </c>
+      <c r="F25">
+        <v>4270</v>
+      </c>
+      <c r="G25">
+        <v>1530</v>
+      </c>
+      <c r="H25">
+        <v>12</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>25</v>
+      </c>
+      <c r="K25">
+        <v>3</v>
+      </c>
+      <c r="L25">
+        <v>16</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>8</v>
+      </c>
+      <c r="P25">
+        <v>4</v>
+      </c>
+      <c r="Q25">
+        <v>69</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0.5</v>
+      </c>
+      <c r="U25">
+        <v>7</v>
+      </c>
+      <c r="V25">
+        <v>6</v>
+      </c>
+      <c r="W25">
+        <v>1</v>
+      </c>
+      <c r="X25">
+        <v>1</v>
+      </c>
+      <c r="Y25">
+        <v>1</v>
+      </c>
+      <c r="Z25">
+        <v>1</v>
+      </c>
+      <c r="AA25">
+        <v>2</v>
+      </c>
+      <c r="AB25">
+        <v>23</v>
+      </c>
+      <c r="AC25">
+        <v>7</v>
+      </c>
+      <c r="AD25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>25/05/2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C26">
+        <v>5770</v>
+      </c>
+      <c r="D26">
+        <v>3830</v>
+      </c>
+      <c r="E26">
+        <v>120</v>
+      </c>
+      <c r="F26">
+        <v>3710</v>
+      </c>
+      <c r="G26">
+        <v>1940</v>
+      </c>
+      <c r="H26">
+        <v>5</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>2</v>
+      </c>
+      <c r="L26">
+        <v>3</v>
+      </c>
+      <c r="M26">
+        <v>2</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>3</v>
+      </c>
+      <c r="P26">
+        <v>3</v>
+      </c>
+      <c r="Q26">
+        <v>18</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <v>1</v>
+      </c>
+      <c r="U26">
+        <v>6</v>
+      </c>
+      <c r="V26">
+        <v>2</v>
+      </c>
+      <c r="W26">
+        <v>2</v>
+      </c>
+      <c r="X26">
+        <v>2</v>
+      </c>
+      <c r="Y26">
+        <v>1.5</v>
+      </c>
+      <c r="Z26">
+        <v>0.5</v>
+      </c>
+      <c r="AA26">
+        <v>10</v>
+      </c>
+      <c r="AB26">
+        <v>9</v>
+      </c>
+      <c r="AC26">
+        <v>8</v>
+      </c>
+      <c r="AD26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>26/05/2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C27">
+        <v>4140</v>
+      </c>
+      <c r="D27">
+        <v>2670</v>
+      </c>
+      <c r="E27">
+        <v>100</v>
+      </c>
+      <c r="F27">
+        <v>2570</v>
+      </c>
+      <c r="G27">
+        <v>1470</v>
+      </c>
+      <c r="H27">
+        <v>15</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>31</v>
+      </c>
+      <c r="K27">
+        <v>3</v>
+      </c>
+      <c r="L27">
+        <v>8</v>
+      </c>
+      <c r="M27">
+        <v>4</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>4</v>
+      </c>
+      <c r="P27">
+        <v>6</v>
+      </c>
+      <c r="Q27">
+        <v>71</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27">
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <v>0.5</v>
+      </c>
+      <c r="U27">
+        <v>6</v>
+      </c>
+      <c r="V27">
+        <v>6</v>
+      </c>
+      <c r="W27">
+        <v>1</v>
+      </c>
+      <c r="X27">
+        <v>1</v>
+      </c>
+      <c r="Y27">
+        <v>0.5</v>
+      </c>
+      <c r="Z27">
+        <v>0.5</v>
+      </c>
+      <c r="AA27">
+        <v>8</v>
+      </c>
+      <c r="AB27">
+        <v>12</v>
+      </c>
+      <c r="AC27">
+        <v>3</v>
+      </c>
+      <c r="AD27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>27/05/2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C28">
+        <v>3840</v>
+      </c>
+      <c r="D28">
+        <v>2840</v>
+      </c>
+      <c r="E28">
+        <v>60</v>
+      </c>
+      <c r="F28">
+        <v>2780</v>
+      </c>
+      <c r="G28">
+        <v>1000</v>
+      </c>
+      <c r="H28">
+        <v>10</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>30</v>
+      </c>
+      <c r="K28">
+        <v>6</v>
+      </c>
+      <c r="L28">
+        <v>8</v>
+      </c>
+      <c r="M28">
+        <v>4</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>4</v>
+      </c>
+      <c r="P28">
+        <v>2</v>
+      </c>
+      <c r="Q28">
+        <v>64</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28">
+        <v>0.5</v>
+      </c>
+      <c r="U28">
+        <v>5</v>
+      </c>
+      <c r="V28">
+        <v>12</v>
+      </c>
+      <c r="W28">
+        <v>0.5</v>
+      </c>
+      <c r="X28">
+        <v>0.5</v>
+      </c>
+      <c r="Y28">
+        <v>0.5</v>
+      </c>
+      <c r="Z28">
+        <v>0.5</v>
+      </c>
+      <c r="AA28">
+        <v>8</v>
+      </c>
+      <c r="AB28">
+        <v>12</v>
+      </c>
+      <c r="AC28">
+        <v>1</v>
+      </c>
+      <c r="AD28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C29">
+        <v>2940</v>
+      </c>
+      <c r="D29">
+        <v>2160</v>
+      </c>
+      <c r="E29">
+        <v>60</v>
+      </c>
+      <c r="F29">
+        <v>2100</v>
+      </c>
+      <c r="G29">
+        <v>780</v>
+      </c>
+      <c r="H29">
+        <v>10</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>5</v>
+      </c>
+      <c r="L29">
+        <v>9</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>3</v>
+      </c>
+      <c r="P29">
+        <v>4</v>
+      </c>
+      <c r="Q29">
+        <v>31</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>0.5</v>
+      </c>
+      <c r="U29">
+        <v>4</v>
+      </c>
+      <c r="V29">
+        <v>10</v>
+      </c>
+      <c r="W29">
+        <v>0</v>
+      </c>
+      <c r="X29">
+        <v>1</v>
+      </c>
+      <c r="Y29">
+        <v>1</v>
+      </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
+      <c r="AA29">
+        <v>0</v>
+      </c>
+      <c r="AB29">
+        <v>6</v>
+      </c>
+      <c r="AC29">
+        <v>5</v>
+      </c>
+      <c r="AD29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C30">
+        <v>7140</v>
+      </c>
+      <c r="D30">
+        <v>3830</v>
+      </c>
+      <c r="E30">
+        <v>120</v>
+      </c>
+      <c r="F30">
+        <v>3710</v>
+      </c>
+      <c r="G30">
+        <v>3310</v>
+      </c>
+      <c r="H30">
+        <v>50</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>7</v>
+      </c>
+      <c r="L30">
+        <v>14</v>
+      </c>
+      <c r="M30">
+        <v>9</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>8</v>
+      </c>
+      <c r="P30">
+        <v>3</v>
+      </c>
+      <c r="Q30">
+        <v>91</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>1</v>
+      </c>
+      <c r="U30">
+        <v>10</v>
+      </c>
+      <c r="V30">
+        <v>14</v>
+      </c>
+      <c r="W30">
+        <v>0.5</v>
+      </c>
+      <c r="X30">
+        <v>0.5</v>
+      </c>
+      <c r="Y30">
+        <v>1</v>
+      </c>
+      <c r="Z30">
+        <v>1</v>
+      </c>
+      <c r="AA30">
+        <v>18</v>
+      </c>
+      <c r="AB30">
+        <v>24</v>
+      </c>
+      <c r="AC30">
+        <v>1.5</v>
+      </c>
+      <c r="AD30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C31">
+        <v>5740</v>
+      </c>
+      <c r="D31">
+        <v>3650</v>
+      </c>
+      <c r="E31">
+        <v>120</v>
+      </c>
+      <c r="F31">
+        <v>3530</v>
+      </c>
+      <c r="G31">
+        <v>2090</v>
+      </c>
+      <c r="H31">
+        <v>18</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>35</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+      <c r="L31">
+        <v>21</v>
+      </c>
+      <c r="M31">
+        <v>5</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>10</v>
+      </c>
+      <c r="P31">
+        <v>3</v>
+      </c>
+      <c r="Q31">
+        <v>97</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>1</v>
+      </c>
+      <c r="U31">
+        <v>3</v>
+      </c>
+      <c r="V31">
+        <v>10</v>
+      </c>
+      <c r="W31">
+        <v>2</v>
+      </c>
+      <c r="X31">
+        <v>2</v>
+      </c>
+      <c r="Y31">
+        <v>1</v>
+      </c>
+      <c r="Z31">
+        <v>1</v>
+      </c>
+      <c r="AA31">
+        <v>10</v>
+      </c>
+      <c r="AB31">
+        <v>30</v>
+      </c>
+      <c r="AC31">
+        <v>2</v>
+      </c>
+      <c r="AD31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>31/05/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C32">
+        <v>4920</v>
+      </c>
+      <c r="D32">
+        <v>2810</v>
+      </c>
+      <c r="E32">
+        <v>90</v>
+      </c>
+      <c r="F32">
+        <v>2720</v>
+      </c>
+      <c r="G32">
+        <v>2110</v>
+      </c>
+      <c r="H32">
+        <v>25</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>30</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32">
+        <v>16</v>
+      </c>
+      <c r="M32">
+        <v>1</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>8</v>
+      </c>
+      <c r="P32">
+        <v>5</v>
+      </c>
+      <c r="Q32">
+        <v>86</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>1</v>
+      </c>
+      <c r="U32">
+        <v>4</v>
+      </c>
+      <c r="V32">
+        <v>2</v>
+      </c>
+      <c r="W32">
+        <v>2</v>
+      </c>
+      <c r="X32">
+        <v>1.5</v>
+      </c>
+      <c r="Y32">
+        <v>1</v>
+      </c>
+      <c r="Z32">
+        <v>1</v>
+      </c>
+      <c r="AA32">
+        <v>2</v>
+      </c>
+      <c r="AB32">
+        <v>24</v>
+      </c>
+      <c r="AC32">
+        <v>3</v>
+      </c>
+      <c r="AD32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B34" t="str">
+        <v>30 days</v>
+      </c>
+      <c r="C34">
+        <v>167381</v>
+      </c>
+      <c r="D34">
+        <v>114241</v>
+      </c>
+      <c r="E34">
+        <v>3160</v>
+      </c>
+      <c r="F34">
+        <v>111081</v>
+      </c>
+      <c r="G34">
+        <v>53140</v>
+      </c>
+      <c r="H34">
+        <v>638</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>790</v>
+      </c>
+      <c r="K34">
+        <v>106</v>
+      </c>
+      <c r="L34">
+        <v>396</v>
+      </c>
+      <c r="M34">
+        <v>139</v>
+      </c>
+      <c r="N34">
+        <v>21</v>
+      </c>
+      <c r="O34">
+        <v>184</v>
+      </c>
+      <c r="P34">
+        <v>180</v>
+      </c>
+      <c r="Q34">
+        <v>2455</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+      <c r="S34">
+        <v>0</v>
+      </c>
+      <c r="T34">
+        <v>127.5</v>
+      </c>
+      <c r="U34">
+        <v>334</v>
+      </c>
+      <c r="V34">
+        <v>184</v>
+      </c>
+      <c r="W34">
+        <v>38.5</v>
+      </c>
+      <c r="X34">
+        <v>41.5</v>
+      </c>
+      <c r="Y34">
+        <v>23</v>
+      </c>
+      <c r="Z34">
+        <v>30</v>
+      </c>
+      <c r="AA34">
+        <v>255</v>
+      </c>
+      <c r="AB34">
+        <v>430</v>
+      </c>
+      <c r="AC34">
+        <v>139.5</v>
+      </c>
+      <c r="AD34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v>AVG/DAY</v>
       </c>
-      <c r="C19">
-        <v>6365.071428571428</v>
-      </c>
-      <c r="D19">
-        <v>4417.214285714285</v>
-      </c>
-      <c r="E19">
-        <v>122.14285714285714</v>
-      </c>
-      <c r="F19">
-        <v>4295.071428571428</v>
-      </c>
-      <c r="G19">
-        <v>1956.4285714285713</v>
-      </c>
-      <c r="H19">
-        <v>38.714285714285715</v>
-      </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
-      <c r="J19">
-        <v>21.714285714285715</v>
-      </c>
-      <c r="K19">
-        <v>59.92857142857143</v>
-      </c>
-      <c r="L19">
-        <v>229.42857142857142</v>
-      </c>
-      <c r="M19">
-        <v>124.71428571428571</v>
-      </c>
-      <c r="N19">
-        <v>33.214285714285715</v>
-      </c>
-      <c r="O19">
-        <v>140.85714285714286</v>
-      </c>
-      <c r="P19">
-        <v>120.14285714285714</v>
-      </c>
-      <c r="Q19">
-        <v>1390.7142857142858</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
-        <v>0</v>
-      </c>
-      <c r="T19">
-        <v>10.142857142857142</v>
-      </c>
-      <c r="U19">
-        <v>21.392857142857142</v>
-      </c>
-      <c r="V19">
-        <v>6.571428571428571</v>
-      </c>
-      <c r="W19">
-        <v>1.4642857142857142</v>
-      </c>
-      <c r="X19">
-        <v>1.7142857142857142</v>
-      </c>
-      <c r="Y19">
-        <v>0.75</v>
-      </c>
-      <c r="Z19">
-        <v>1.3214285714285714</v>
-      </c>
-      <c r="AA19">
-        <v>9.5</v>
-      </c>
-      <c r="AB19">
-        <v>12.071428571428571</v>
-      </c>
-      <c r="AC19">
-        <v>7</v>
-      </c>
-      <c r="AD19">
-        <v>2</v>
+      <c r="C35">
+        <v>5579.366666666667</v>
+      </c>
+      <c r="D35">
+        <v>3808.0333333333333</v>
+      </c>
+      <c r="E35">
+        <v>105.33333333333333</v>
+      </c>
+      <c r="F35">
+        <v>3702.7</v>
+      </c>
+      <c r="G35">
+        <v>1771.3333333333333</v>
+      </c>
+      <c r="H35">
+        <v>21.266666666666666</v>
+      </c>
+      <c r="I35">
+        <v>0.03333333333333333</v>
+      </c>
+      <c r="J35">
+        <v>26.333333333333332</v>
+      </c>
+      <c r="K35">
+        <v>3.533333333333333</v>
+      </c>
+      <c r="L35">
+        <v>13.2</v>
+      </c>
+      <c r="M35">
+        <v>4.633333333333334</v>
+      </c>
+      <c r="N35">
+        <v>0.7</v>
+      </c>
+      <c r="O35">
+        <v>6.133333333333334</v>
+      </c>
+      <c r="P35">
+        <v>6</v>
+      </c>
+      <c r="Q35">
+        <v>81.83333333333333</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <v>4.25</v>
+      </c>
+      <c r="U35">
+        <v>11.133333333333333</v>
+      </c>
+      <c r="V35">
+        <v>6.133333333333334</v>
+      </c>
+      <c r="W35">
+        <v>1.2833333333333334</v>
+      </c>
+      <c r="X35">
+        <v>1.3833333333333333</v>
+      </c>
+      <c r="Y35">
+        <v>0.7666666666666667</v>
+      </c>
+      <c r="Z35">
+        <v>1</v>
+      </c>
+      <c r="AA35">
+        <v>8.5</v>
+      </c>
+      <c r="AB35">
+        <v>14.333333333333334</v>
+      </c>
+      <c r="AC35">
+        <v>4.65</v>
+      </c>
+      <c r="AD35">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: resolve mobile layout issue with full-width header column flex, bump version to v3.2.2
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1197,22 +1197,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>01/01/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>May26</v>
+        <v>Apr26</v>
       </c>
       <c r="C4" t="str">
         <v>OPEX</v>
       </c>
       <c r="D4" t="str">
-        <v>Fixed Costs</v>
+        <v>Salary</v>
       </c>
       <c r="E4" t="str">
-        <v>ค่าเช่าร้าน 2 เดือนพฤษภาคม</v>
+        <v>Employee 3</v>
       </c>
       <c r="F4">
-        <v>30000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="5">
@@ -1229,10 +1229,10 @@
         <v>Salary</v>
       </c>
       <c r="E5" t="str">
-        <v>Employee 3</v>
+        <v>Employee 4</v>
       </c>
       <c r="F5">
-        <v>12000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="6">
@@ -1246,13 +1246,13 @@
         <v>OPEX</v>
       </c>
       <c r="D6" t="str">
-        <v>Salary</v>
+        <v>Fixed Costs</v>
       </c>
       <c r="E6" t="str">
-        <v>Employee 4</v>
+        <v>Rent</v>
       </c>
       <c r="F6">
-        <v>6000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="7">
@@ -1266,33 +1266,33 @@
         <v>OPEX</v>
       </c>
       <c r="D7" t="str">
-        <v>Fixed Costs</v>
+        <v>Investment</v>
       </c>
       <c r="E7" t="str">
-        <v>Rent</v>
+        <v>Stock (Allocated 17.1%)</v>
       </c>
       <c r="F7">
-        <v>30000</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>30/04/2026</v>
+        <v>07/05/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>Apr26</v>
+        <v>May26</v>
       </c>
       <c r="C8" t="str">
         <v>OPEX</v>
       </c>
       <c r="D8" t="str">
-        <v>Investment</v>
+        <v>Rental</v>
       </c>
       <c r="E8" t="str">
-        <v>Stock (Allocated 17.1%)</v>
+        <v>ค่าเช่าร้าน 2 เดือนพฤษภาคม</v>
       </c>
       <c r="F8">
-        <v>2052</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="9">
@@ -1355,9 +1355,29 @@
         <v>4830</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>01/06/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C12" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E12" t="str">
+        <v>ค่าที่ร้านน้ำส้ม b2 06/26</v>
+      </c>
+      <c r="F12">
+        <v>30000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3298,16 +3318,16 @@
         <v>6570</v>
       </c>
       <c r="D6">
-        <v>4950</v>
+        <v>5070</v>
       </c>
       <c r="E6">
         <v>120</v>
       </c>
       <c r="F6">
-        <v>4830</v>
+        <v>4950</v>
       </c>
       <c r="G6">
-        <v>1620</v>
+        <v>1500</v>
       </c>
       <c r="H6">
         <v>23</v>
@@ -3316,7 +3336,7 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -3337,7 +3357,7 @@
         <v>9</v>
       </c>
       <c r="Q6">
-        <v>67</v>
+        <v>113</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -3770,34 +3790,34 @@
         <v>2160</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="K11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N11">
         <v>0</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -3862,13 +3882,13 @@
         <v>1440</v>
       </c>
       <c r="H12">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="K12">
         <v>4</v>
@@ -3883,13 +3903,13 @@
         <v>1</v>
       </c>
       <c r="O12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P12">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="Q12">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -4043,22 +4063,22 @@
         <v>2430</v>
       </c>
       <c r="G14">
-        <v>850</v>
+        <v>970</v>
       </c>
       <c r="H14">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K14">
         <v>1</v>
       </c>
       <c r="L14">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M14">
         <v>10</v>
@@ -4070,10 +4090,10 @@
         <v>8</v>
       </c>
       <c r="P14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q14">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="R14">
         <v>0</v>
@@ -4690,13 +4710,13 @@
         <v>450</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="I21">
         <v>0</v>
       </c>
       <c r="J21">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K21">
         <v>2</v>
@@ -4717,7 +4737,7 @@
         <v>2</v>
       </c>
       <c r="Q21">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="R21">
         <v>0</v>
@@ -4874,16 +4894,16 @@
         <v>1720</v>
       </c>
       <c r="H23">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="K23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L23">
         <v>10</v>
@@ -4895,13 +4915,13 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P23">
         <v>10</v>
       </c>
       <c r="Q23">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="R23">
         <v>0</v>
@@ -5058,13 +5078,13 @@
         <v>1530</v>
       </c>
       <c r="H25">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I25">
         <v>0</v>
       </c>
       <c r="J25">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="K25">
         <v>3</v>
@@ -5073,7 +5093,7 @@
         <v>16</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -5082,10 +5102,10 @@
         <v>8</v>
       </c>
       <c r="P25">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="Q25">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="R25">
         <v>0</v>
@@ -5150,22 +5170,22 @@
         <v>1940</v>
       </c>
       <c r="H26">
+        <v>17</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>38</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <v>21</v>
+      </c>
+      <c r="M26">
         <v>5</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26">
-        <v>2</v>
-      </c>
-      <c r="L26">
-        <v>3</v>
-      </c>
-      <c r="M26">
-        <v>2</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -5174,10 +5194,10 @@
         <v>3</v>
       </c>
       <c r="P26">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="Q26">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="R26">
         <v>0</v>
@@ -5432,7 +5452,7 @@
         <v>0</v>
       </c>
       <c r="J29">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="K29">
         <v>5</v>
@@ -5453,7 +5473,7 @@
         <v>4</v>
       </c>
       <c r="Q29">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="R29">
         <v>0</v>
@@ -5518,13 +5538,13 @@
         <v>3310</v>
       </c>
       <c r="H30">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I30">
         <v>0</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="K30">
         <v>7</v>
@@ -5545,7 +5565,7 @@
         <v>3</v>
       </c>
       <c r="Q30">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="R30">
         <v>0</v>
@@ -5961,72 +5981,1577 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AD19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Som Sai Jai Cold Press Bar - June 2026</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Revenue (฿)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Cash (฿)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Expenses (฿)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Cash-Exp (฿)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Scan/Transfer (฿)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Orange</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Watermelon</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Coconut</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Apple</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Young Coco</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Total Cups</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Bot Big</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Bot Small</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Used Orange (basket)</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Used Watermelon (pcs)</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Used Young Coco</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Date</v>
+        <v>01/06/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>Day</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Revenue (฿)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Cash (฿)</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Expenses (฿)</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Cash-Exp (฿)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Scan/Transfer (฿)</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Orange</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Watermelon</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Mango</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Coconut</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Apple</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Young Coco</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Total Cups</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Bot Big</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Bot Small</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Used Orange (basket)</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Used Watermelon (pcs)</v>
+        <v>Mon</v>
+      </c>
+      <c r="C3">
+        <v>5860</v>
+      </c>
+      <c r="D3">
+        <v>4220</v>
+      </c>
+      <c r="E3">
+        <v>120</v>
+      </c>
+      <c r="F3">
+        <v>4100</v>
+      </c>
+      <c r="G3">
+        <v>1640</v>
+      </c>
+      <c r="H3">
+        <v>18</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>35</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>12</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="P3">
+        <v>17</v>
+      </c>
+      <c r="Q3">
+        <v>98</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0.5</v>
+      </c>
+      <c r="U3">
+        <v>8</v>
+      </c>
+      <c r="V3">
+        <v>10</v>
+      </c>
+      <c r="W3">
+        <v>1.5</v>
+      </c>
+      <c r="X3">
+        <v>1.5</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>10</v>
+      </c>
+      <c r="AB3">
+        <v>7</v>
+      </c>
+      <c r="AC3">
+        <v>9</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>02/06/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C4">
+        <v>4120</v>
+      </c>
+      <c r="D4">
+        <v>2610</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <v>2550</v>
+      </c>
+      <c r="G4">
+        <v>1510</v>
+      </c>
+      <c r="H4">
+        <v>9</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>41</v>
+      </c>
+      <c r="K4">
+        <v>5</v>
+      </c>
+      <c r="L4">
+        <v>8</v>
+      </c>
+      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>2</v>
+      </c>
+      <c r="P4">
+        <v>3</v>
+      </c>
+      <c r="Q4">
+        <v>72</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0.5</v>
+      </c>
+      <c r="U4">
+        <v>8</v>
+      </c>
+      <c r="V4">
+        <v>10</v>
+      </c>
+      <c r="W4">
+        <v>0.5</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0.5</v>
+      </c>
+      <c r="AA4">
+        <v>8</v>
+      </c>
+      <c r="AB4">
+        <v>3</v>
+      </c>
+      <c r="AC4">
+        <v>2</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>03/06/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C5">
+        <v>5210</v>
+      </c>
+      <c r="D5">
+        <v>2860</v>
+      </c>
+      <c r="E5">
+        <v>120</v>
+      </c>
+      <c r="F5">
+        <v>2740</v>
+      </c>
+      <c r="G5">
+        <v>2350</v>
+      </c>
+      <c r="H5">
+        <v>19</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>8</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>21</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>13</v>
+      </c>
+      <c r="P5">
+        <v>13</v>
+      </c>
+      <c r="Q5">
+        <v>91</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>18</v>
+      </c>
+      <c r="U5">
+        <v>36</v>
+      </c>
+      <c r="V5">
+        <v>2</v>
+      </c>
+      <c r="W5">
+        <v>1.5</v>
+      </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>1</v>
+      </c>
+      <c r="AA5">
+        <v>7</v>
+      </c>
+      <c r="AB5">
+        <v>10</v>
+      </c>
+      <c r="AC5">
+        <v>7</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>04/06/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C6">
+        <v>3680</v>
+      </c>
+      <c r="D6">
+        <v>2020</v>
+      </c>
+      <c r="E6">
+        <v>120</v>
+      </c>
+      <c r="F6">
+        <v>1900</v>
+      </c>
+      <c r="G6">
+        <v>1660</v>
+      </c>
+      <c r="H6">
+        <v>28</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>31</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>66</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>1.5</v>
+      </c>
+      <c r="U6">
+        <v>6</v>
+      </c>
+      <c r="V6">
+        <v>2</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>8</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>05/06/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C7">
+        <v>5880</v>
+      </c>
+      <c r="D7">
+        <v>4140</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="F7">
+        <v>4080</v>
+      </c>
+      <c r="G7">
+        <v>1740</v>
+      </c>
+      <c r="H7">
+        <v>21</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>21</v>
+      </c>
+      <c r="K7">
+        <v>5</v>
+      </c>
+      <c r="L7">
+        <v>23</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>6</v>
+      </c>
+      <c r="P7">
+        <v>13</v>
+      </c>
+      <c r="Q7">
+        <v>99</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>1.5</v>
+      </c>
+      <c r="U7">
+        <v>5</v>
+      </c>
+      <c r="V7">
+        <v>10</v>
+      </c>
+      <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7">
+        <v>1</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7">
+        <v>8</v>
+      </c>
+      <c r="AB7">
+        <v>18</v>
+      </c>
+      <c r="AC7">
+        <v>9</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>06/06/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C8">
+        <v>4950</v>
+      </c>
+      <c r="D8">
+        <v>2640</v>
+      </c>
+      <c r="E8">
+        <v>120</v>
+      </c>
+      <c r="F8">
+        <v>2400</v>
+      </c>
+      <c r="G8">
+        <v>2310</v>
+      </c>
+      <c r="H8">
+        <v>18</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>36</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <v>10</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>5</v>
+      </c>
+      <c r="P8">
+        <v>4</v>
+      </c>
+      <c r="Q8">
+        <v>82</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0.5</v>
+      </c>
+      <c r="U8">
+        <v>6</v>
+      </c>
+      <c r="V8">
+        <v>10</v>
+      </c>
+      <c r="W8">
+        <v>1</v>
+      </c>
+      <c r="X8">
+        <v>1</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>8</v>
+      </c>
+      <c r="AB8">
+        <v>15</v>
+      </c>
+      <c r="AC8">
+        <v>2</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>07/06/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C9">
+        <v>4000</v>
+      </c>
+      <c r="D9">
+        <v>2440</v>
+      </c>
+      <c r="E9">
+        <v>120</v>
+      </c>
+      <c r="F9">
+        <v>2320</v>
+      </c>
+      <c r="G9">
+        <v>1560</v>
+      </c>
+      <c r="H9">
+        <v>13</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>26</v>
+      </c>
+      <c r="K9">
+        <v>2</v>
+      </c>
+      <c r="L9">
+        <v>16</v>
+      </c>
+      <c r="M9">
+        <v>3</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>6</v>
+      </c>
+      <c r="P9">
+        <v>2</v>
+      </c>
+      <c r="Q9">
+        <v>68</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0.5</v>
+      </c>
+      <c r="U9">
+        <v>4</v>
+      </c>
+      <c r="V9">
+        <v>4</v>
+      </c>
+      <c r="W9">
+        <v>1</v>
+      </c>
+      <c r="X9">
+        <v>1.5</v>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9">
+        <v>1</v>
+      </c>
+      <c r="AA9">
+        <v>6</v>
+      </c>
+      <c r="AB9">
+        <v>18</v>
+      </c>
+      <c r="AC9">
+        <v>2</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>08/06/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C10">
+        <v>3380</v>
+      </c>
+      <c r="D10">
+        <v>2210</v>
+      </c>
+      <c r="E10">
+        <v>90</v>
+      </c>
+      <c r="F10">
+        <v>2120</v>
+      </c>
+      <c r="G10">
+        <v>1170</v>
+      </c>
+      <c r="H10">
+        <v>14</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>16</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>11</v>
+      </c>
+      <c r="M10">
+        <v>6</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>2</v>
+      </c>
+      <c r="P10">
+        <v>7</v>
+      </c>
+      <c r="Q10">
+        <v>57</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0.5</v>
+      </c>
+      <c r="U10">
+        <v>4</v>
+      </c>
+      <c r="V10">
+        <v>2</v>
+      </c>
+      <c r="W10">
+        <v>1</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10">
+        <v>1</v>
+      </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
+        <v>12</v>
+      </c>
+      <c r="AB10">
+        <v>6</v>
+      </c>
+      <c r="AC10">
+        <v>4</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>09/06/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C11">
+        <v>2860</v>
+      </c>
+      <c r="D11">
+        <v>1910</v>
+      </c>
+      <c r="E11">
+        <v>60</v>
+      </c>
+      <c r="F11">
+        <v>1850</v>
+      </c>
+      <c r="G11">
+        <v>950</v>
+      </c>
+      <c r="H11">
+        <v>15</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>14</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <v>9</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>2</v>
+      </c>
+      <c r="P11">
+        <v>7</v>
+      </c>
+      <c r="Q11">
+        <v>49</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>1.5</v>
+      </c>
+      <c r="U11">
+        <v>4</v>
+      </c>
+      <c r="V11">
+        <v>1</v>
+      </c>
+      <c r="W11">
+        <v>1</v>
+      </c>
+      <c r="X11">
+        <v>1</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>1</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>6</v>
+      </c>
+      <c r="AC11">
+        <v>4</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>10/06/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C12">
+        <v>2840</v>
+      </c>
+      <c r="D12">
+        <v>1980</v>
+      </c>
+      <c r="E12">
+        <v>60</v>
+      </c>
+      <c r="F12">
+        <v>1920</v>
+      </c>
+      <c r="G12">
+        <v>860</v>
+      </c>
+      <c r="H12">
+        <v>9</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>28</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>8</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>2</v>
+      </c>
+      <c r="P12">
+        <v>2</v>
+      </c>
+      <c r="Q12">
+        <v>50</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0.5</v>
+      </c>
+      <c r="U12">
+        <v>4</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>1</v>
+      </c>
+      <c r="X12">
+        <v>0.5</v>
+      </c>
+      <c r="Y12">
+        <v>1</v>
+      </c>
+      <c r="Z12">
+        <v>1</v>
+      </c>
+      <c r="AA12">
+        <v>2</v>
+      </c>
+      <c r="AB12">
+        <v>12</v>
+      </c>
+      <c r="AC12">
+        <v>1</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>11/06/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C13">
+        <v>2290</v>
+      </c>
+      <c r="D13">
+        <v>1500</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="F13">
+        <v>1440</v>
+      </c>
+      <c r="G13">
+        <v>790</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>10</v>
+      </c>
+      <c r="K13">
+        <v>3</v>
+      </c>
+      <c r="L13">
+        <v>10</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>7</v>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13">
+        <v>34</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0.5</v>
+      </c>
+      <c r="U13">
+        <v>2</v>
+      </c>
+      <c r="V13">
+        <v>6</v>
+      </c>
+      <c r="W13">
+        <v>0.5</v>
+      </c>
+      <c r="X13">
+        <v>0.5</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>2</v>
+      </c>
+      <c r="AB13">
+        <v>2</v>
+      </c>
+      <c r="AC13">
+        <v>0.5</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>13/06/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C14">
+        <v>7530</v>
+      </c>
+      <c r="D14">
+        <v>4380</v>
+      </c>
+      <c r="E14">
+        <v>120</v>
+      </c>
+      <c r="F14">
+        <v>4260</v>
+      </c>
+      <c r="G14">
+        <v>3150</v>
+      </c>
+      <c r="H14">
+        <v>22</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>50</v>
+      </c>
+      <c r="K14">
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <v>27</v>
+      </c>
+      <c r="M14">
+        <v>6</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>8</v>
+      </c>
+      <c r="P14">
+        <v>12</v>
+      </c>
+      <c r="Q14">
+        <v>130</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>1</v>
+      </c>
+      <c r="U14">
+        <v>4</v>
+      </c>
+      <c r="V14">
+        <v>10</v>
+      </c>
+      <c r="W14">
+        <v>2.5</v>
+      </c>
+      <c r="X14">
+        <v>2</v>
+      </c>
+      <c r="Y14">
+        <v>1</v>
+      </c>
+      <c r="Z14">
+        <v>1</v>
+      </c>
+      <c r="AA14">
+        <v>12</v>
+      </c>
+      <c r="AB14">
+        <v>24</v>
+      </c>
+      <c r="AC14">
+        <v>6</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>14/06/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C15">
+        <v>5090</v>
+      </c>
+      <c r="D15">
+        <v>3560</v>
+      </c>
+      <c r="E15">
+        <v>90</v>
+      </c>
+      <c r="F15">
+        <v>3470</v>
+      </c>
+      <c r="G15">
+        <v>1530</v>
+      </c>
+      <c r="H15">
+        <v>16</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>33</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+      <c r="L15">
+        <v>18</v>
+      </c>
+      <c r="M15">
+        <v>4</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>4</v>
+      </c>
+      <c r="P15">
+        <v>6</v>
+      </c>
+      <c r="Q15">
+        <v>84</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15">
+        <v>5</v>
+      </c>
+      <c r="V15">
+        <v>6</v>
+      </c>
+      <c r="W15">
+        <v>1</v>
+      </c>
+      <c r="X15">
+        <v>1.5</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15">
+        <v>1</v>
+      </c>
+      <c r="AA15">
+        <v>8</v>
+      </c>
+      <c r="AB15">
+        <v>12</v>
+      </c>
+      <c r="AC15">
+        <v>3</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>12/6/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C16">
+        <v>1400</v>
+      </c>
+      <c r="D16">
+        <v>1020</v>
+      </c>
+      <c r="E16">
+        <v>60</v>
+      </c>
+      <c r="F16">
+        <v>960</v>
+      </c>
+      <c r="G16">
+        <v>380</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>4</v>
+      </c>
+      <c r="K16">
+        <v>2</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16">
+        <v>4</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>3</v>
+      </c>
+      <c r="Q16">
+        <v>23</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0.5</v>
+      </c>
+      <c r="U16">
+        <v>1</v>
+      </c>
+      <c r="V16">
+        <v>4</v>
+      </c>
+      <c r="W16">
+        <v>0.5</v>
+      </c>
+      <c r="X16">
+        <v>0.5</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>8</v>
+      </c>
+      <c r="AB16">
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <v>2</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B18" t="str">
+        <v>13 days</v>
+      </c>
+      <c r="C18">
+        <v>53230</v>
+      </c>
+      <c r="D18">
+        <v>33150</v>
+      </c>
+      <c r="E18">
+        <v>1140</v>
+      </c>
+      <c r="F18">
+        <v>32010</v>
+      </c>
+      <c r="G18">
+        <v>20080</v>
+      </c>
+      <c r="H18">
+        <v>796</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>189</v>
+      </c>
+      <c r="K18">
+        <v>932</v>
+      </c>
+      <c r="L18">
+        <v>1217</v>
+      </c>
+      <c r="M18">
+        <v>556</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>457</v>
+      </c>
+      <c r="P18">
+        <v>489</v>
+      </c>
+      <c r="Q18">
+        <v>4636</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>124.5</v>
+      </c>
+      <c r="U18">
+        <v>200</v>
+      </c>
+      <c r="V18">
+        <v>57</v>
+      </c>
+      <c r="W18">
+        <v>14.5</v>
+      </c>
+      <c r="X18">
+        <v>12.5</v>
+      </c>
+      <c r="Y18">
+        <v>6</v>
+      </c>
+      <c r="Z18">
+        <v>8.5</v>
+      </c>
+      <c r="AA18">
+        <v>86</v>
+      </c>
+      <c r="AB18">
+        <v>117</v>
+      </c>
+      <c r="AC18">
+        <v>45.5</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>AVG/DAY</v>
+      </c>
+      <c r="C19">
+        <v>4094.6153846153848</v>
+      </c>
+      <c r="D19">
+        <v>2550</v>
+      </c>
+      <c r="E19">
+        <v>87.6923076923077</v>
+      </c>
+      <c r="F19">
+        <v>2462.3076923076924</v>
+      </c>
+      <c r="G19">
+        <v>1544.6153846153845</v>
+      </c>
+      <c r="H19">
+        <v>61.23076923076923</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>14.538461538461538</v>
+      </c>
+      <c r="K19">
+        <v>71.6923076923077</v>
+      </c>
+      <c r="L19">
+        <v>93.61538461538461</v>
+      </c>
+      <c r="M19">
+        <v>42.76923076923077</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>35.15384615384615</v>
+      </c>
+      <c r="P19">
+        <v>37.61538461538461</v>
+      </c>
+      <c r="Q19">
+        <v>356.61538461538464</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>9.576923076923077</v>
+      </c>
+      <c r="U19">
+        <v>15.384615384615385</v>
+      </c>
+      <c r="V19">
+        <v>4.384615384615385</v>
+      </c>
+      <c r="W19">
+        <v>1.1153846153846154</v>
+      </c>
+      <c r="X19">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="Y19">
+        <v>0.46153846153846156</v>
+      </c>
+      <c r="Z19">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="AA19">
+        <v>6.615384615384615</v>
+      </c>
+      <c r="AB19">
+        <v>9</v>
+      </c>
+      <c r="AC19">
+        <v>3.5</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: correct B2 orange-usage data-entry bug across 7 days (May-Jun26)
Found that on specific days, the "orange baskets used" field in B2 sales
reports had the cup-sold count typed in instead of the actual basket
count (verified against source report images for all 7 dates: 09, 14,
16, 17, 19, 22 May and 03 June). This inflated B2's usage-based share of
the shared Orange COGS allocation by ~101 phantom basket-units, dragging
down B2's reported May/June net profit. Corrected using each day's real
usage value from the handwritten "Stock" section of the sales sheet.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
@@ -3886,7 +3886,7 @@
         <v>0</v>
       </c>
       <c r="T11">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="U11">
         <v>35</v>
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="T16">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="U16">
         <v>11</v>
@@ -4530,7 +4530,7 @@
         <v>0</v>
       </c>
       <c r="T18">
-        <v>14</v>
+        <v>0.5</v>
       </c>
       <c r="U18">
         <v>31</v>
@@ -4622,7 +4622,7 @@
         <v>0</v>
       </c>
       <c r="T19">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="U19">
         <v>29</v>
@@ -4806,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="T21">
-        <v>9</v>
+        <v>0.5</v>
       </c>
       <c r="U21">
         <v>23</v>
@@ -4990,7 +4990,7 @@
         <v>0</v>
       </c>
       <c r="T23">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="U23">
         <v>4</v>
@@ -6383,7 +6383,7 @@
         <v>0</v>
       </c>
       <c r="T5">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="U5">
         <v>36</v>

</xml_diff>

<commit_message>
feat: effective-dated profit share, B3 onboarding, and complete ice audit
profitShareFor(branch, month) replaces the static PROFIT_SHARE_RATIO map so
B1's Jul26 transition from 60/40 to 70/30 applies going forward without
rewriting the rate already paid on closed months (business_rules.js,
index.html sharePct()). Also adds daily_exp (cash paid at the stall, mostly
ice) as its own P&L line rather than folding it into net silently.

Onboards B3 (Platinum Pop) as a full branch across data.json,
reports_data.json, and the B3 Excel, with docs (CLAUDE.md/AGENTS.md/GEMINI.md)
updated to match.

Finishes the ice expense audit (ice_audit.json): B2/Jul26 was the last
outstanding month (31/31 days) — every day's ice value re-verified against
that sheet's own cash-minus-ice arithmetic and confirmed already correct in
the ledger, so apply_ice_audit.js applied zero corrections.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B2_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1435,9 +1435,129 @@
         <v>6000</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>22/07/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Jul26</v>
+      </c>
+      <c r="C16" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Salary b2 wei 20days 450/day (LINE_ALBUM_Cost July_260802_72.jpg)</v>
+      </c>
+      <c r="F16">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Jul26</v>
+      </c>
+      <c r="C17" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Rent B2</v>
+      </c>
+      <c r="F17">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Jul26</v>
+      </c>
+      <c r="C18" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Salary B2 (Remaining)</v>
+      </c>
+      <c r="F18">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>06/07/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Jul26</v>
+      </c>
+      <c r="C19" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E19" t="str">
+        <v>ค่าเช่า stock เดือน june (1/3 split B2)</v>
+      </c>
+      <c r="F19">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>31/05/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C20" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E20" t="str">
+        <v>ปรับปรุงเงินเดือน พ.ค. (ยืนยัน 17,200)</v>
+      </c>
+      <c r="F20">
+        <v>-800</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>14/05/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C21" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E21" t="str">
+        <v>ค่าเช่า stock พ.ค. (B2 ครึ่งหนึ่ง)</v>
+      </c>
+      <c r="F21">
+        <v>6000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1895,10 +2015,10 @@
         <v>1120</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F4">
-        <v>1120</v>
+        <v>1060</v>
       </c>
       <c r="G4">
         <v>1190</v>
@@ -2455,10 +2575,10 @@
         <v>3950</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F11">
-        <v>3950</v>
+        <v>3890</v>
       </c>
       <c r="G11">
         <v>1820</v>
@@ -2615,10 +2735,10 @@
         <v>3140</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F13">
-        <v>3140</v>
+        <v>3020</v>
       </c>
       <c r="G13">
         <v>1520</v>
@@ -2992,7 +3112,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD35"/>
+  <dimension ref="A1:AD36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3841,10 +3961,10 @@
         <v>3601</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F11">
-        <v>3601</v>
+        <v>3481</v>
       </c>
       <c r="G11">
         <v>2160</v>
@@ -4933,40 +5053,40 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>22/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C23">
-        <v>5660</v>
+        <v>4150</v>
       </c>
       <c r="D23">
-        <v>3940</v>
+        <v>2300</v>
       </c>
       <c r="E23">
         <v>120</v>
       </c>
       <c r="F23">
-        <v>3820</v>
+        <v>2180</v>
       </c>
       <c r="G23">
-        <v>1720</v>
+        <v>1850</v>
       </c>
       <c r="H23">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="J23">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="K23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L23">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M23">
         <v>5</v>
@@ -4975,49 +5095,49 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="P23">
+        <v>3</v>
+      </c>
+      <c r="Q23">
+        <v>70</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0.5</v>
+      </c>
+      <c r="U23">
+        <v>6</v>
+      </c>
+      <c r="V23">
+        <v>6</v>
+      </c>
+      <c r="W23">
+        <v>1</v>
+      </c>
+      <c r="X23">
+        <v>1</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
         <v>10</v>
       </c>
-      <c r="Q23">
-        <v>98</v>
-      </c>
-      <c r="R23">
-        <v>0</v>
-      </c>
-      <c r="S23">
-        <v>0</v>
-      </c>
-      <c r="T23">
-        <v>1</v>
-      </c>
-      <c r="U23">
-        <v>4</v>
-      </c>
-      <c r="V23">
-        <v>4</v>
-      </c>
-      <c r="W23">
-        <v>1</v>
-      </c>
-      <c r="X23">
-        <v>1</v>
-      </c>
-      <c r="Y23">
-        <v>1</v>
-      </c>
-      <c r="Z23">
-        <v>1</v>
-      </c>
-      <c r="AA23">
-        <v>5</v>
-      </c>
       <c r="AB23">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AC23">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AD23">
         <v>0</v>
@@ -5025,43 +5145,43 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>23/05/2026</v>
+        <v>22/05/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>Sat</v>
+        <v>Fri</v>
       </c>
       <c r="C24">
-        <v>5740</v>
+        <v>5660</v>
       </c>
       <c r="D24">
-        <v>3260</v>
+        <v>3940</v>
       </c>
       <c r="E24">
         <v>120</v>
       </c>
       <c r="F24">
-        <v>3140</v>
+        <v>3820</v>
       </c>
       <c r="G24">
-        <v>2480</v>
+        <v>1720</v>
       </c>
       <c r="H24">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="J24">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="K24">
         <v>4</v>
       </c>
       <c r="L24">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -5070,46 +5190,46 @@
         <v>7</v>
       </c>
       <c r="P24">
+        <v>10</v>
+      </c>
+      <c r="Q24">
+        <v>98</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>1</v>
+      </c>
+      <c r="U24">
         <v>4</v>
       </c>
-      <c r="Q24">
-        <v>100</v>
-      </c>
-      <c r="R24">
-        <v>0</v>
-      </c>
-      <c r="S24">
-        <v>0</v>
-      </c>
-      <c r="T24">
-        <v>1</v>
-      </c>
-      <c r="U24">
+      <c r="V24">
+        <v>4</v>
+      </c>
+      <c r="W24">
+        <v>1</v>
+      </c>
+      <c r="X24">
+        <v>1</v>
+      </c>
+      <c r="Y24">
+        <v>1</v>
+      </c>
+      <c r="Z24">
+        <v>1</v>
+      </c>
+      <c r="AA24">
+        <v>5</v>
+      </c>
+      <c r="AB24">
         <v>7</v>
       </c>
-      <c r="V24">
-        <v>8</v>
-      </c>
-      <c r="W24">
-        <v>1</v>
-      </c>
-      <c r="X24">
-        <v>1</v>
-      </c>
-      <c r="Y24">
-        <v>1</v>
-      </c>
-      <c r="Z24">
-        <v>1</v>
-      </c>
-      <c r="AA24">
-        <v>12</v>
-      </c>
-      <c r="AB24">
-        <v>21</v>
-      </c>
       <c r="AC24">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AD24">
         <v>0</v>
@@ -5117,55 +5237,55 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>24/05/2026</v>
+        <v>23/05/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>Sun</v>
+        <v>Sat</v>
       </c>
       <c r="C25">
-        <v>5920</v>
+        <v>5740</v>
       </c>
       <c r="D25">
-        <v>4390</v>
+        <v>3260</v>
       </c>
       <c r="E25">
         <v>120</v>
       </c>
       <c r="F25">
-        <v>4270</v>
+        <v>3140</v>
       </c>
       <c r="G25">
-        <v>1530</v>
+        <v>2480</v>
       </c>
       <c r="H25">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="I25">
         <v>0</v>
       </c>
       <c r="J25">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="K25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L25">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="M25">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N25">
         <v>0</v>
       </c>
       <c r="O25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P25">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="Q25">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="R25">
         <v>0</v>
@@ -5174,13 +5294,13 @@
         <v>0</v>
       </c>
       <c r="T25">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U25">
         <v>7</v>
       </c>
       <c r="V25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W25">
         <v>1</v>
@@ -5195,13 +5315,13 @@
         <v>1</v>
       </c>
       <c r="AA25">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="AB25">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AC25">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AD25">
         <v>0</v>
@@ -5209,55 +5329,55 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>25/05/2026</v>
+        <v>24/05/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>Mon</v>
+        <v>Sun</v>
       </c>
       <c r="C26">
-        <v>5770</v>
+        <v>5920</v>
       </c>
       <c r="D26">
-        <v>3830</v>
+        <v>4390</v>
       </c>
       <c r="E26">
         <v>120</v>
       </c>
       <c r="F26">
-        <v>3710</v>
+        <v>4270</v>
       </c>
       <c r="G26">
-        <v>1940</v>
+        <v>1530</v>
       </c>
       <c r="H26">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I26">
         <v>0</v>
       </c>
       <c r="J26">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L26">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N26">
         <v>0</v>
       </c>
       <c r="O26">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="P26">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q26">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="R26">
         <v>0</v>
@@ -5266,34 +5386,34 @@
         <v>0</v>
       </c>
       <c r="T26">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="U26">
+        <v>7</v>
+      </c>
+      <c r="V26">
         <v>6</v>
       </c>
-      <c r="V26">
-        <v>2</v>
-      </c>
       <c r="W26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y26">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="Z26">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AA26">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AB26">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="AC26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AD26">
         <v>0</v>
@@ -5301,56 +5421,56 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>26/05/2026</v>
+        <v>25/05/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>Tue</v>
+        <v>Mon</v>
       </c>
       <c r="C27">
-        <v>4140</v>
+        <v>5770</v>
       </c>
       <c r="D27">
-        <v>2670</v>
+        <v>3830</v>
       </c>
       <c r="E27">
+        <v>120</v>
+      </c>
+      <c r="F27">
+        <v>3710</v>
+      </c>
+      <c r="G27">
+        <v>1940</v>
+      </c>
+      <c r="H27">
+        <v>17</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>38</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="L27">
+        <v>21</v>
+      </c>
+      <c r="M27">
+        <v>5</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>3</v>
+      </c>
+      <c r="P27">
+        <v>15</v>
+      </c>
+      <c r="Q27">
         <v>100</v>
       </c>
-      <c r="F27">
-        <v>2570</v>
-      </c>
-      <c r="G27">
-        <v>1470</v>
-      </c>
-      <c r="H27">
-        <v>15</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>31</v>
-      </c>
-      <c r="K27">
-        <v>3</v>
-      </c>
-      <c r="L27">
-        <v>8</v>
-      </c>
-      <c r="M27">
-        <v>4</v>
-      </c>
-      <c r="N27">
-        <v>0</v>
-      </c>
-      <c r="O27">
-        <v>4</v>
-      </c>
-      <c r="P27">
-        <v>6</v>
-      </c>
-      <c r="Q27">
-        <v>71</v>
-      </c>
       <c r="R27">
         <v>0</v>
       </c>
@@ -5358,34 +5478,34 @@
         <v>0</v>
       </c>
       <c r="T27">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U27">
         <v>6</v>
       </c>
       <c r="V27">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y27">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="Z27">
         <v>0.5</v>
       </c>
       <c r="AA27">
+        <v>10</v>
+      </c>
+      <c r="AB27">
+        <v>9</v>
+      </c>
+      <c r="AC27">
         <v>8</v>
-      </c>
-      <c r="AB27">
-        <v>12</v>
-      </c>
-      <c r="AC27">
-        <v>3</v>
       </c>
       <c r="AD27">
         <v>0</v>
@@ -5393,37 +5513,37 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>27/05/2026</v>
+        <v>26/05/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>Wed</v>
+        <v>Tue</v>
       </c>
       <c r="C28">
-        <v>3840</v>
+        <v>4140</v>
       </c>
       <c r="D28">
-        <v>2840</v>
+        <v>2670</v>
       </c>
       <c r="E28">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="F28">
-        <v>2780</v>
+        <v>2570</v>
       </c>
       <c r="G28">
-        <v>1000</v>
+        <v>1470</v>
       </c>
       <c r="H28">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="J28">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K28">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L28">
         <v>8</v>
@@ -5438,10 +5558,10 @@
         <v>4</v>
       </c>
       <c r="P28">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q28">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="R28">
         <v>0</v>
@@ -5453,16 +5573,16 @@
         <v>0.5</v>
       </c>
       <c r="U28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V28">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="W28">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="X28">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="Y28">
         <v>0.5</v>
@@ -5477,7 +5597,7 @@
         <v>12</v>
       </c>
       <c r="AC28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD28">
         <v>0</v>
@@ -5485,25 +5605,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>28/05/2026</v>
+        <v>27/05/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>Thu</v>
+        <v>Wed</v>
       </c>
       <c r="C29">
-        <v>2940</v>
+        <v>3840</v>
       </c>
       <c r="D29">
-        <v>2160</v>
+        <v>2840</v>
       </c>
       <c r="E29">
         <v>60</v>
       </c>
       <c r="F29">
-        <v>2100</v>
+        <v>2780</v>
       </c>
       <c r="G29">
-        <v>780</v>
+        <v>1000</v>
       </c>
       <c r="H29">
         <v>10</v>
@@ -5512,28 +5632,28 @@
         <v>0</v>
       </c>
       <c r="J29">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M29">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N29">
         <v>0</v>
       </c>
       <c r="O29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q29">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="R29">
         <v>0</v>
@@ -5545,31 +5665,31 @@
         <v>0.5</v>
       </c>
       <c r="U29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V29">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W29">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="X29">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Y29">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Z29">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AA29">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AB29">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="AC29">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD29">
         <v>0</v>
@@ -5577,55 +5697,55 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>29/05/2026</v>
+        <v>28/05/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>Fri</v>
+        <v>Thu</v>
       </c>
       <c r="C30">
-        <v>7140</v>
+        <v>2940</v>
       </c>
       <c r="D30">
-        <v>3830</v>
+        <v>2160</v>
       </c>
       <c r="E30">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F30">
-        <v>3710</v>
+        <v>2100</v>
       </c>
       <c r="G30">
-        <v>3310</v>
+        <v>780</v>
       </c>
       <c r="H30">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="I30">
         <v>0</v>
       </c>
       <c r="J30">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="K30">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L30">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M30">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N30">
         <v>0</v>
       </c>
       <c r="O30">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="P30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q30">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="R30">
         <v>0</v>
@@ -5634,34 +5754,34 @@
         <v>0</v>
       </c>
       <c r="T30">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="U30">
+        <v>4</v>
+      </c>
+      <c r="V30">
         <v>10</v>
       </c>
-      <c r="V30">
-        <v>14</v>
-      </c>
       <c r="W30">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="X30">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="Y30">
         <v>1</v>
       </c>
       <c r="Z30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA30">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="AB30">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="AC30">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="AD30">
         <v>0</v>
@@ -5669,55 +5789,55 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>30/05/2026</v>
+        <v>29/05/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>Sat</v>
+        <v>Fri</v>
       </c>
       <c r="C31">
-        <v>5740</v>
+        <v>7140</v>
       </c>
       <c r="D31">
-        <v>3650</v>
+        <v>3830</v>
       </c>
       <c r="E31">
         <v>120</v>
       </c>
       <c r="F31">
-        <v>3530</v>
+        <v>3710</v>
       </c>
       <c r="G31">
-        <v>2090</v>
+        <v>3310</v>
       </c>
       <c r="H31">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I31">
         <v>0</v>
       </c>
       <c r="J31">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L31">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N31">
         <v>0</v>
       </c>
       <c r="O31">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P31">
         <v>3</v>
       </c>
       <c r="Q31">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="R31">
         <v>0</v>
@@ -5729,16 +5849,16 @@
         <v>1</v>
       </c>
       <c r="U31">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="V31">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="W31">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="X31">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="Y31">
         <v>1</v>
@@ -5747,13 +5867,13 @@
         <v>1</v>
       </c>
       <c r="AA31">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="AB31">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="AC31">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="AD31">
         <v>0</v>
@@ -5761,280 +5881,372 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
+        <v>30/05/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C32">
+        <v>5740</v>
+      </c>
+      <c r="D32">
+        <v>3650</v>
+      </c>
+      <c r="E32">
+        <v>120</v>
+      </c>
+      <c r="F32">
+        <v>3530</v>
+      </c>
+      <c r="G32">
+        <v>2090</v>
+      </c>
+      <c r="H32">
+        <v>18</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>35</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+      <c r="L32">
+        <v>21</v>
+      </c>
+      <c r="M32">
+        <v>5</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>10</v>
+      </c>
+      <c r="P32">
+        <v>3</v>
+      </c>
+      <c r="Q32">
+        <v>97</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>1</v>
+      </c>
+      <c r="U32">
+        <v>3</v>
+      </c>
+      <c r="V32">
+        <v>10</v>
+      </c>
+      <c r="W32">
+        <v>2</v>
+      </c>
+      <c r="X32">
+        <v>2</v>
+      </c>
+      <c r="Y32">
+        <v>1</v>
+      </c>
+      <c r="Z32">
+        <v>1</v>
+      </c>
+      <c r="AA32">
+        <v>10</v>
+      </c>
+      <c r="AB32">
+        <v>30</v>
+      </c>
+      <c r="AC32">
+        <v>2</v>
+      </c>
+      <c r="AD32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
         <v>31/05/2026</v>
       </c>
-      <c r="B32" t="str">
+      <c r="B33" t="str">
         <v>Sun</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>4920</v>
       </c>
-      <c r="D32">
+      <c r="D33">
         <v>2810</v>
       </c>
-      <c r="E32">
+      <c r="E33">
         <v>90</v>
       </c>
-      <c r="F32">
+      <c r="F33">
         <v>2720</v>
       </c>
-      <c r="G32">
+      <c r="G33">
         <v>2110</v>
       </c>
-      <c r="H32">
+      <c r="H33">
         <v>25</v>
       </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
-      <c r="J32">
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
         <v>30</v>
       </c>
-      <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="L32">
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
         <v>16</v>
       </c>
-      <c r="M32">
-        <v>1</v>
-      </c>
-      <c r="N32">
-        <v>0</v>
-      </c>
-      <c r="O32">
+      <c r="M33">
+        <v>1</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
         <v>8</v>
       </c>
-      <c r="P32">
+      <c r="P33">
         <v>5</v>
       </c>
-      <c r="Q32">
+      <c r="Q33">
         <v>86</v>
       </c>
-      <c r="R32">
-        <v>0</v>
-      </c>
-      <c r="S32">
-        <v>0</v>
-      </c>
-      <c r="T32">
-        <v>1</v>
-      </c>
-      <c r="U32">
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>1</v>
+      </c>
+      <c r="U33">
         <v>4</v>
       </c>
-      <c r="V32">
-        <v>2</v>
-      </c>
-      <c r="W32">
-        <v>2</v>
-      </c>
-      <c r="X32">
+      <c r="V33">
+        <v>2</v>
+      </c>
+      <c r="W33">
+        <v>2</v>
+      </c>
+      <c r="X33">
         <v>1.5</v>
       </c>
-      <c r="Y32">
-        <v>1</v>
-      </c>
-      <c r="Z32">
-        <v>1</v>
-      </c>
-      <c r="AA32">
-        <v>2</v>
-      </c>
-      <c r="AB32">
+      <c r="Y33">
+        <v>1</v>
+      </c>
+      <c r="Z33">
+        <v>1</v>
+      </c>
+      <c r="AA33">
+        <v>2</v>
+      </c>
+      <c r="AB33">
         <v>24</v>
       </c>
-      <c r="AC32">
+      <c r="AC33">
         <v>3</v>
       </c>
-      <c r="AD32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B34" t="str">
-        <v>30 days</v>
-      </c>
-      <c r="C34">
-        <v>167381</v>
-      </c>
-      <c r="D34">
-        <v>114361</v>
-      </c>
-      <c r="E34">
-        <v>3160</v>
-      </c>
-      <c r="F34">
-        <v>111201</v>
-      </c>
-      <c r="G34">
-        <v>53140</v>
-      </c>
-      <c r="H34">
-        <v>635</v>
-      </c>
-      <c r="I34">
-        <v>1</v>
-      </c>
-      <c r="J34">
-        <v>1118</v>
-      </c>
-      <c r="K34">
-        <v>108</v>
-      </c>
-      <c r="L34">
-        <v>437</v>
-      </c>
-      <c r="M34">
-        <v>148</v>
-      </c>
-      <c r="N34">
-        <v>21</v>
-      </c>
-      <c r="O34">
-        <v>189</v>
-      </c>
-      <c r="P34">
-        <v>219</v>
-      </c>
-      <c r="Q34">
-        <v>2878</v>
-      </c>
-      <c r="R34">
-        <v>0</v>
-      </c>
-      <c r="S34">
-        <v>0</v>
-      </c>
-      <c r="T34">
-        <v>127.5</v>
-      </c>
-      <c r="U34">
-        <v>334</v>
-      </c>
-      <c r="V34">
-        <v>184</v>
-      </c>
-      <c r="W34">
-        <v>38.5</v>
-      </c>
-      <c r="X34">
-        <v>41.5</v>
-      </c>
-      <c r="Y34">
-        <v>23</v>
-      </c>
-      <c r="Z34">
-        <v>30</v>
-      </c>
-      <c r="AA34">
-        <v>255</v>
-      </c>
-      <c r="AB34">
-        <v>430</v>
-      </c>
-      <c r="AC34">
-        <v>139.5</v>
-      </c>
-      <c r="AD34">
+      <c r="AD33">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B35" t="str">
+        <v>31 days</v>
+      </c>
+      <c r="C35">
+        <v>171531</v>
+      </c>
+      <c r="D35">
+        <v>116661</v>
+      </c>
+      <c r="E35">
+        <v>3280</v>
+      </c>
+      <c r="F35">
+        <v>113381</v>
+      </c>
+      <c r="G35">
+        <v>54990</v>
+      </c>
+      <c r="H35">
+        <v>653</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>1145</v>
+      </c>
+      <c r="K35">
+        <v>113</v>
+      </c>
+      <c r="L35">
+        <v>448</v>
+      </c>
+      <c r="M35">
+        <v>153</v>
+      </c>
+      <c r="N35">
+        <v>21</v>
+      </c>
+      <c r="O35">
+        <v>190</v>
+      </c>
+      <c r="P35">
+        <v>222</v>
+      </c>
+      <c r="Q35">
+        <v>2948</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <v>33</v>
+      </c>
+      <c r="U35">
+        <v>340</v>
+      </c>
+      <c r="V35">
+        <v>190</v>
+      </c>
+      <c r="W35">
+        <v>39.5</v>
+      </c>
+      <c r="X35">
+        <v>42.5</v>
+      </c>
+      <c r="Y35">
+        <v>23</v>
+      </c>
+      <c r="Z35">
+        <v>30</v>
+      </c>
+      <c r="AA35">
+        <v>265</v>
+      </c>
+      <c r="AB35">
+        <v>433</v>
+      </c>
+      <c r="AC35">
+        <v>140.5</v>
+      </c>
+      <c r="AD35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>AVG/DAY</v>
       </c>
-      <c r="C35">
-        <v>5579.366666666667</v>
-      </c>
-      <c r="D35">
-        <v>3812.0333333333333</v>
-      </c>
-      <c r="E35">
-        <v>105.33333333333333</v>
-      </c>
-      <c r="F35">
-        <v>3706.7</v>
-      </c>
-      <c r="G35">
-        <v>1771.3333333333333</v>
-      </c>
-      <c r="H35">
-        <v>21.166666666666668</v>
-      </c>
-      <c r="I35">
-        <v>0.03333333333333333</v>
-      </c>
-      <c r="J35">
-        <v>37.266666666666666</v>
-      </c>
-      <c r="K35">
-        <v>3.6</v>
-      </c>
-      <c r="L35">
-        <v>14.566666666666666</v>
-      </c>
-      <c r="M35">
-        <v>4.933333333333334</v>
-      </c>
-      <c r="N35">
-        <v>0.7</v>
-      </c>
-      <c r="O35">
-        <v>6.3</v>
-      </c>
-      <c r="P35">
-        <v>7.3</v>
-      </c>
-      <c r="Q35">
-        <v>95.93333333333334</v>
-      </c>
-      <c r="R35">
-        <v>0</v>
-      </c>
-      <c r="S35">
-        <v>0</v>
-      </c>
-      <c r="T35">
-        <v>4.25</v>
-      </c>
-      <c r="U35">
-        <v>11.133333333333333</v>
-      </c>
-      <c r="V35">
-        <v>6.133333333333334</v>
-      </c>
-      <c r="W35">
-        <v>1.2833333333333334</v>
-      </c>
-      <c r="X35">
-        <v>1.3833333333333333</v>
-      </c>
-      <c r="Y35">
-        <v>0.7666666666666667</v>
-      </c>
-      <c r="Z35">
-        <v>1</v>
-      </c>
-      <c r="AA35">
-        <v>8.5</v>
-      </c>
-      <c r="AB35">
-        <v>14.333333333333334</v>
-      </c>
-      <c r="AC35">
-        <v>4.65</v>
-      </c>
-      <c r="AD35">
+      <c r="C36">
+        <v>5533.258064516129</v>
+      </c>
+      <c r="D36">
+        <v>3763.2580645161293</v>
+      </c>
+      <c r="E36">
+        <v>105.80645161290323</v>
+      </c>
+      <c r="F36">
+        <v>3657.451612903226</v>
+      </c>
+      <c r="G36">
+        <v>1773.8709677419354</v>
+      </c>
+      <c r="H36">
+        <v>21.06451612903226</v>
+      </c>
+      <c r="I36">
+        <v>0.03225806451612903</v>
+      </c>
+      <c r="J36">
+        <v>36.935483870967744</v>
+      </c>
+      <c r="K36">
+        <v>3.6451612903225805</v>
+      </c>
+      <c r="L36">
+        <v>14.451612903225806</v>
+      </c>
+      <c r="M36">
+        <v>4.935483870967742</v>
+      </c>
+      <c r="N36">
+        <v>0.6774193548387096</v>
+      </c>
+      <c r="O36">
+        <v>6.129032258064516</v>
+      </c>
+      <c r="P36">
+        <v>7.161290322580645</v>
+      </c>
+      <c r="Q36">
+        <v>95.09677419354838</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+      <c r="S36">
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <v>1.064516129032258</v>
+      </c>
+      <c r="U36">
+        <v>10.96774193548387</v>
+      </c>
+      <c r="V36">
+        <v>6.129032258064516</v>
+      </c>
+      <c r="W36">
+        <v>1.2741935483870968</v>
+      </c>
+      <c r="X36">
+        <v>1.3709677419354838</v>
+      </c>
+      <c r="Y36">
+        <v>0.7419354838709677</v>
+      </c>
+      <c r="Z36">
+        <v>0.967741935483871</v>
+      </c>
+      <c r="AA36">
+        <v>8.548387096774194</v>
+      </c>
+      <c r="AB36">
+        <v>13.96774193548387</v>
+      </c>
+      <c r="AC36">
+        <v>4.532258064516129</v>
+      </c>
+      <c r="AD36">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7534,10 +7746,10 @@
         <v>4540</v>
       </c>
       <c r="E18">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F18">
-        <v>4420</v>
+        <v>4480</v>
       </c>
       <c r="G18">
         <v>1110</v>
@@ -9090,72 +9302,2960 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AD33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Som Sai Jai Cold Press Bar - July 2026</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Revenue (฿)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Cash (฿)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Expenses (฿)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Cash-Exp (฿)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Scan/Transfer (฿)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Orange</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Watermelon</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Coconut</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Apple</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Young Coco</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Total Cups</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Bot Big</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Bot Small</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Used Orange (basket)</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Used Watermelon (pcs)</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Used Young Coco</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Date</v>
+        <v>01/07/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>Day</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Revenue (฿)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Cash (฿)</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Expenses (฿)</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Cash-Exp (฿)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Scan/Transfer (฿)</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Orange</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Watermelon</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Mango</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Coconut</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Apple</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Young Coco</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Total Cups</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Bot Big</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Bot Small</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Used Orange (basket)</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Used Watermelon (pcs)</v>
+        <v>Wed</v>
+      </c>
+      <c r="C3">
+        <v>5200</v>
+      </c>
+      <c r="D3">
+        <v>3010</v>
+      </c>
+      <c r="E3">
+        <v>60</v>
+      </c>
+      <c r="F3">
+        <v>2950</v>
+      </c>
+      <c r="G3">
+        <v>2190</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>42</v>
+      </c>
+      <c r="K3">
+        <v>7</v>
+      </c>
+      <c r="L3">
+        <v>14</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>7</v>
+      </c>
+      <c r="P3">
+        <v>7</v>
+      </c>
+      <c r="Q3">
+        <v>89</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3">
+        <v>7</v>
+      </c>
+      <c r="V3">
+        <v>10</v>
+      </c>
+      <c r="W3">
+        <v>1</v>
+      </c>
+      <c r="X3">
+        <v>1</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="Z3">
+        <v>1</v>
+      </c>
+      <c r="AA3">
+        <v>13</v>
+      </c>
+      <c r="AB3">
+        <v>20</v>
+      </c>
+      <c r="AC3">
+        <v>3</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>02/07/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C4">
+        <v>410</v>
+      </c>
+      <c r="D4">
+        <v>220</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <v>160</v>
+      </c>
+      <c r="G4">
+        <v>190</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>7</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>1</v>
+      </c>
+      <c r="U4">
+        <v>2</v>
+      </c>
+      <c r="V4">
+        <v>5</v>
+      </c>
+      <c r="W4">
+        <v>4</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>10</v>
+      </c>
+      <c r="AB4">
+        <v>15</v>
+      </c>
+      <c r="AC4">
+        <v>1</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>03/07/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C5">
+        <v>6960</v>
+      </c>
+      <c r="D5">
+        <v>5020</v>
+      </c>
+      <c r="E5">
+        <v>60</v>
+      </c>
+      <c r="F5">
+        <v>4960</v>
+      </c>
+      <c r="G5">
+        <v>1940</v>
+      </c>
+      <c r="H5">
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>63</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>5</v>
+      </c>
+      <c r="P5">
+        <v>6</v>
+      </c>
+      <c r="Q5">
+        <v>116</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>1</v>
+      </c>
+      <c r="U5">
+        <v>7</v>
+      </c>
+      <c r="V5">
+        <v>5</v>
+      </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>1</v>
+      </c>
+      <c r="Z5">
+        <v>1</v>
+      </c>
+      <c r="AA5">
+        <v>10</v>
+      </c>
+      <c r="AB5">
+        <v>10</v>
+      </c>
+      <c r="AC5">
+        <v>7</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>04/07/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C6">
+        <v>5200</v>
+      </c>
+      <c r="D6">
+        <v>3000</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>2940</v>
+      </c>
+      <c r="G6">
+        <v>2200</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>40</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>15</v>
+      </c>
+      <c r="M6">
+        <v>5</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>6</v>
+      </c>
+      <c r="P6">
+        <v>5</v>
+      </c>
+      <c r="Q6">
+        <v>86</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <v>6</v>
+      </c>
+      <c r="V6">
+        <v>8</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6">
+        <v>1</v>
+      </c>
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6">
+        <v>1</v>
+      </c>
+      <c r="AA6">
+        <v>12</v>
+      </c>
+      <c r="AB6">
+        <v>15</v>
+      </c>
+      <c r="AC6">
+        <v>4</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>05/07/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C7">
+        <v>3550</v>
+      </c>
+      <c r="D7">
+        <v>2270</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="F7">
+        <v>2210</v>
+      </c>
+      <c r="G7">
+        <v>1280</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>26</v>
+      </c>
+      <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>7</v>
+      </c>
+      <c r="P7">
+        <v>7</v>
+      </c>
+      <c r="Q7">
+        <v>58</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>1</v>
+      </c>
+      <c r="U7">
+        <v>4</v>
+      </c>
+      <c r="V7">
+        <v>10</v>
+      </c>
+      <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7">
+        <v>1</v>
+      </c>
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7">
+        <v>10</v>
+      </c>
+      <c r="AB7">
+        <v>25</v>
+      </c>
+      <c r="AC7">
+        <v>4</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>06/07/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C8">
+        <v>3730</v>
+      </c>
+      <c r="D8">
+        <v>2820</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="F8">
+        <v>2760</v>
+      </c>
+      <c r="G8">
+        <v>910</v>
+      </c>
+      <c r="H8">
+        <v>7</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>32</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="L8">
+        <v>13</v>
+      </c>
+      <c r="M8">
+        <v>2</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>7</v>
+      </c>
+      <c r="P8">
+        <v>4</v>
+      </c>
+      <c r="Q8">
+        <v>67</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="U8">
+        <v>6</v>
+      </c>
+      <c r="V8">
+        <v>5</v>
+      </c>
+      <c r="W8">
+        <v>1</v>
+      </c>
+      <c r="X8">
+        <v>1</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8">
+        <v>1</v>
+      </c>
+      <c r="AA8">
+        <v>10</v>
+      </c>
+      <c r="AB8">
+        <v>20</v>
+      </c>
+      <c r="AC8">
+        <v>5</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>07/07/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C9">
+        <v>3030</v>
+      </c>
+      <c r="D9">
+        <v>2360</v>
+      </c>
+      <c r="E9">
+        <v>60</v>
+      </c>
+      <c r="F9">
+        <v>2300</v>
+      </c>
+      <c r="G9">
+        <v>670</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>25</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>14</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>2</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9">
+        <v>52</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>4</v>
+      </c>
+      <c r="U9">
+        <v>5</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0.5</v>
+      </c>
+      <c r="X9">
+        <v>0.5</v>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9">
+        <v>1</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
+        <v>6</v>
+      </c>
+      <c r="AC9">
+        <v>0.5</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>08/07/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C10">
+        <v>2300</v>
+      </c>
+      <c r="D10">
+        <v>1470</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="F10">
+        <v>1410</v>
+      </c>
+      <c r="G10">
+        <v>830</v>
+      </c>
+      <c r="H10">
+        <v>5</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>22</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>6</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>40</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>1</v>
+      </c>
+      <c r="U10">
+        <v>3</v>
+      </c>
+      <c r="V10">
+        <v>10</v>
+      </c>
+      <c r="W10">
+        <v>1</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>10</v>
+      </c>
+      <c r="AB10">
+        <v>15</v>
+      </c>
+      <c r="AC10">
+        <v>3</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>09/07/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C11">
+        <v>4490</v>
+      </c>
+      <c r="D11">
+        <v>3250</v>
+      </c>
+      <c r="E11">
+        <v>60</v>
+      </c>
+      <c r="F11">
+        <v>3190</v>
+      </c>
+      <c r="G11">
+        <v>1240</v>
+      </c>
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>30</v>
+      </c>
+      <c r="K11">
+        <v>9</v>
+      </c>
+      <c r="L11">
+        <v>17</v>
+      </c>
+      <c r="M11">
+        <v>3</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>3</v>
+      </c>
+      <c r="P11">
+        <v>4</v>
+      </c>
+      <c r="Q11">
+        <v>74</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <v>3</v>
+      </c>
+      <c r="V11">
+        <v>9.5</v>
+      </c>
+      <c r="W11">
+        <v>2</v>
+      </c>
+      <c r="X11">
+        <v>2</v>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+      <c r="Z11">
+        <v>1</v>
+      </c>
+      <c r="AA11">
+        <v>10</v>
+      </c>
+      <c r="AB11">
+        <v>15</v>
+      </c>
+      <c r="AC11">
+        <v>5</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>10/07/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C12">
+        <v>5030</v>
+      </c>
+      <c r="D12">
+        <v>3330</v>
+      </c>
+      <c r="E12">
+        <v>60</v>
+      </c>
+      <c r="F12">
+        <v>3270</v>
+      </c>
+      <c r="G12">
+        <v>1700</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>32</v>
+      </c>
+      <c r="K12">
+        <v>7</v>
+      </c>
+      <c r="L12">
+        <v>23</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>10</v>
+      </c>
+      <c r="P12">
+        <v>2</v>
+      </c>
+      <c r="Q12">
+        <v>84</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>2</v>
+      </c>
+      <c r="U12">
+        <v>4</v>
+      </c>
+      <c r="V12">
+        <v>10</v>
+      </c>
+      <c r="W12">
+        <v>2</v>
+      </c>
+      <c r="X12">
+        <v>2</v>
+      </c>
+      <c r="Y12">
+        <v>1</v>
+      </c>
+      <c r="Z12">
+        <v>1</v>
+      </c>
+      <c r="AA12">
+        <v>10</v>
+      </c>
+      <c r="AB12">
+        <v>25</v>
+      </c>
+      <c r="AC12">
+        <v>3</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>11/07/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C13">
+        <v>4890</v>
+      </c>
+      <c r="D13">
+        <v>2860</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="F13">
+        <v>2800</v>
+      </c>
+      <c r="G13">
+        <v>2030</v>
+      </c>
+      <c r="H13">
+        <v>11</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>22</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+      <c r="L13">
+        <v>16</v>
+      </c>
+      <c r="M13">
+        <v>11</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>5</v>
+      </c>
+      <c r="P13">
+        <v>4</v>
+      </c>
+      <c r="Q13">
+        <v>73</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>1</v>
+      </c>
+      <c r="U13">
+        <v>3</v>
+      </c>
+      <c r="V13">
+        <v>5</v>
+      </c>
+      <c r="W13">
+        <v>2</v>
+      </c>
+      <c r="X13">
+        <v>2</v>
+      </c>
+      <c r="Y13">
+        <v>1</v>
+      </c>
+      <c r="Z13">
+        <v>0.5</v>
+      </c>
+      <c r="AA13">
+        <v>25</v>
+      </c>
+      <c r="AB13">
+        <v>30</v>
+      </c>
+      <c r="AC13">
+        <v>5</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>12/07/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C14">
+        <v>5070</v>
+      </c>
+      <c r="D14">
+        <v>3070</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="F14">
+        <v>3010</v>
+      </c>
+      <c r="G14">
+        <v>2000</v>
+      </c>
+      <c r="H14">
+        <v>12</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>42</v>
+      </c>
+      <c r="K14">
+        <v>3</v>
+      </c>
+      <c r="L14">
+        <v>10</v>
+      </c>
+      <c r="M14">
+        <v>3</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>9</v>
+      </c>
+      <c r="P14">
+        <v>9</v>
+      </c>
+      <c r="Q14">
+        <v>88</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>1</v>
+      </c>
+      <c r="U14">
+        <v>5</v>
+      </c>
+      <c r="V14">
+        <v>9</v>
+      </c>
+      <c r="W14">
+        <v>2</v>
+      </c>
+      <c r="X14">
+        <v>2</v>
+      </c>
+      <c r="Y14">
+        <v>1</v>
+      </c>
+      <c r="Z14">
+        <v>1</v>
+      </c>
+      <c r="AA14">
+        <v>20</v>
+      </c>
+      <c r="AB14">
+        <v>20</v>
+      </c>
+      <c r="AC14">
+        <v>5</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>13/07/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C15">
+        <v>3350</v>
+      </c>
+      <c r="D15">
+        <v>2300</v>
+      </c>
+      <c r="E15">
+        <v>60</v>
+      </c>
+      <c r="F15">
+        <v>2240</v>
+      </c>
+      <c r="G15">
+        <v>1050</v>
+      </c>
+      <c r="H15">
+        <v>5</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>19</v>
+      </c>
+      <c r="K15">
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <v>16</v>
+      </c>
+      <c r="M15">
+        <v>7</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>4</v>
+      </c>
+      <c r="P15">
+        <v>3</v>
+      </c>
+      <c r="Q15">
+        <v>58</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0.5</v>
+      </c>
+      <c r="U15">
+        <v>5</v>
+      </c>
+      <c r="V15">
+        <v>10</v>
+      </c>
+      <c r="W15">
+        <v>2</v>
+      </c>
+      <c r="X15">
+        <v>2</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15">
+        <v>2</v>
+      </c>
+      <c r="AA15">
+        <v>20</v>
+      </c>
+      <c r="AB15">
+        <v>32</v>
+      </c>
+      <c r="AC15">
+        <v>4</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C16">
+        <v>4000</v>
+      </c>
+      <c r="D16">
+        <v>2790</v>
+      </c>
+      <c r="E16">
+        <v>60</v>
+      </c>
+      <c r="F16">
+        <v>2730</v>
+      </c>
+      <c r="G16">
+        <v>1210</v>
+      </c>
+      <c r="H16">
+        <v>7</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>24</v>
+      </c>
+      <c r="K16">
+        <v>5</v>
+      </c>
+      <c r="L16">
+        <v>14</v>
+      </c>
+      <c r="M16">
+        <v>5</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>9</v>
+      </c>
+      <c r="P16">
+        <v>3</v>
+      </c>
+      <c r="Q16">
+        <v>67</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>1</v>
+      </c>
+      <c r="U16">
+        <v>4</v>
+      </c>
+      <c r="V16">
+        <v>10</v>
+      </c>
+      <c r="W16">
+        <v>2</v>
+      </c>
+      <c r="X16">
+        <v>2</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>10</v>
+      </c>
+      <c r="AB16">
+        <v>27</v>
+      </c>
+      <c r="AC16">
+        <v>5</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C17">
+        <v>4470</v>
+      </c>
+      <c r="D17">
+        <v>3250</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="F17">
+        <v>3190</v>
+      </c>
+      <c r="G17">
+        <v>1220</v>
+      </c>
+      <c r="H17">
+        <v>10</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>31</v>
+      </c>
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <v>13</v>
+      </c>
+      <c r="M17">
+        <v>7</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>4</v>
+      </c>
+      <c r="P17">
+        <v>7</v>
+      </c>
+      <c r="Q17">
+        <v>76</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>4</v>
+      </c>
+      <c r="V17">
+        <v>5</v>
+      </c>
+      <c r="W17">
+        <v>1</v>
+      </c>
+      <c r="X17">
+        <v>1</v>
+      </c>
+      <c r="Y17">
+        <v>1</v>
+      </c>
+      <c r="Z17">
+        <v>1</v>
+      </c>
+      <c r="AA17">
+        <v>20</v>
+      </c>
+      <c r="AB17">
+        <v>15</v>
+      </c>
+      <c r="AC17">
+        <v>5</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>16/07/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C18">
+        <v>1970</v>
+      </c>
+      <c r="D18">
+        <v>1450</v>
+      </c>
+      <c r="E18">
+        <v>60</v>
+      </c>
+      <c r="F18">
+        <v>1390</v>
+      </c>
+      <c r="G18">
+        <v>520</v>
+      </c>
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>12</v>
+      </c>
+      <c r="K18">
+        <v>6</v>
+      </c>
+      <c r="L18">
+        <v>2</v>
+      </c>
+      <c r="M18">
+        <v>4</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
+        <v>1</v>
+      </c>
+      <c r="Q18">
+        <v>31</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>1</v>
+      </c>
+      <c r="U18">
+        <v>3</v>
+      </c>
+      <c r="V18">
+        <v>10</v>
+      </c>
+      <c r="W18">
+        <v>1</v>
+      </c>
+      <c r="X18">
+        <v>1</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>10</v>
+      </c>
+      <c r="AB18">
+        <v>10</v>
+      </c>
+      <c r="AC18">
+        <v>3</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>17/07/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C19">
+        <v>5450</v>
+      </c>
+      <c r="D19">
+        <v>3910</v>
+      </c>
+      <c r="E19">
+        <v>60</v>
+      </c>
+      <c r="F19">
+        <v>3850</v>
+      </c>
+      <c r="G19">
+        <v>1540</v>
+      </c>
+      <c r="H19">
+        <v>8</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>42</v>
+      </c>
+      <c r="K19">
+        <v>7</v>
+      </c>
+      <c r="L19">
+        <v>14</v>
+      </c>
+      <c r="M19">
+        <v>8</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>6</v>
+      </c>
+      <c r="P19">
+        <v>8</v>
+      </c>
+      <c r="Q19">
+        <v>93</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0.5</v>
+      </c>
+      <c r="U19">
+        <v>20</v>
+      </c>
+      <c r="V19">
+        <v>15</v>
+      </c>
+      <c r="W19">
+        <v>1</v>
+      </c>
+      <c r="X19">
+        <v>1</v>
+      </c>
+      <c r="Y19">
+        <v>1</v>
+      </c>
+      <c r="Z19">
+        <v>1</v>
+      </c>
+      <c r="AA19">
+        <v>15</v>
+      </c>
+      <c r="AB19">
+        <v>20</v>
+      </c>
+      <c r="AC19">
+        <v>6</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>18/07/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C20">
+        <v>6170</v>
+      </c>
+      <c r="D20">
+        <v>3430</v>
+      </c>
+      <c r="E20">
+        <v>90</v>
+      </c>
+      <c r="F20">
+        <v>3340</v>
+      </c>
+      <c r="G20">
+        <v>2740</v>
+      </c>
+      <c r="H20">
+        <v>17</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>34</v>
+      </c>
+      <c r="K20">
+        <v>4</v>
+      </c>
+      <c r="L20">
+        <v>13</v>
+      </c>
+      <c r="M20">
+        <v>11</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>10</v>
+      </c>
+      <c r="P20">
+        <v>10</v>
+      </c>
+      <c r="Q20">
+        <v>99</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>1</v>
+      </c>
+      <c r="U20">
+        <v>5</v>
+      </c>
+      <c r="V20">
+        <v>4</v>
+      </c>
+      <c r="W20">
+        <v>1</v>
+      </c>
+      <c r="X20">
+        <v>1</v>
+      </c>
+      <c r="Y20">
+        <v>1</v>
+      </c>
+      <c r="Z20">
+        <v>1</v>
+      </c>
+      <c r="AA20">
+        <v>20</v>
+      </c>
+      <c r="AB20">
+        <v>10</v>
+      </c>
+      <c r="AC20">
+        <v>4</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>19/07/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C21">
+        <v>5040</v>
+      </c>
+      <c r="D21">
+        <v>3280</v>
+      </c>
+      <c r="E21">
+        <v>120</v>
+      </c>
+      <c r="F21">
+        <v>3160</v>
+      </c>
+      <c r="G21">
+        <v>1760</v>
+      </c>
+      <c r="H21">
+        <v>13</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>32</v>
+      </c>
+      <c r="K21">
+        <v>4</v>
+      </c>
+      <c r="L21">
+        <v>9</v>
+      </c>
+      <c r="M21">
+        <v>11</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>9</v>
+      </c>
+      <c r="P21">
+        <v>10</v>
+      </c>
+      <c r="Q21">
+        <v>88</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>1</v>
+      </c>
+      <c r="U21">
+        <v>5</v>
+      </c>
+      <c r="V21">
+        <v>4</v>
+      </c>
+      <c r="W21">
+        <v>1</v>
+      </c>
+      <c r="X21">
+        <v>1</v>
+      </c>
+      <c r="Y21">
+        <v>0.5</v>
+      </c>
+      <c r="Z21">
+        <v>0.5</v>
+      </c>
+      <c r="AA21">
+        <v>20</v>
+      </c>
+      <c r="AB21">
+        <v>10</v>
+      </c>
+      <c r="AC21">
+        <v>4</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>20/07/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C22">
+        <v>6800</v>
+      </c>
+      <c r="D22">
+        <v>5190</v>
+      </c>
+      <c r="E22">
+        <v>120</v>
+      </c>
+      <c r="F22">
+        <v>5070</v>
+      </c>
+      <c r="G22">
+        <v>1610</v>
+      </c>
+      <c r="H22">
+        <v>16</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>32</v>
+      </c>
+      <c r="K22">
+        <v>10</v>
+      </c>
+      <c r="L22">
+        <v>24</v>
+      </c>
+      <c r="M22">
+        <v>7</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>15</v>
+      </c>
+      <c r="P22">
+        <v>5</v>
+      </c>
+      <c r="Q22">
+        <v>109</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>0.5</v>
+      </c>
+      <c r="U22">
+        <v>5</v>
+      </c>
+      <c r="V22">
+        <v>20</v>
+      </c>
+      <c r="W22">
+        <v>1</v>
+      </c>
+      <c r="X22">
+        <v>0.5</v>
+      </c>
+      <c r="Y22">
+        <v>1</v>
+      </c>
+      <c r="Z22">
+        <v>1</v>
+      </c>
+      <c r="AA22">
+        <v>14</v>
+      </c>
+      <c r="AB22">
+        <v>90</v>
+      </c>
+      <c r="AC22">
+        <v>3.5</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>21/07/2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C23">
+        <v>5640</v>
+      </c>
+      <c r="D23">
+        <v>3800</v>
+      </c>
+      <c r="E23">
+        <v>60</v>
+      </c>
+      <c r="F23">
+        <v>3740</v>
+      </c>
+      <c r="G23">
+        <v>1840</v>
+      </c>
+      <c r="H23">
+        <v>14</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>41</v>
+      </c>
+      <c r="K23">
+        <v>3</v>
+      </c>
+      <c r="L23">
+        <v>14</v>
+      </c>
+      <c r="M23">
+        <v>4</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>9</v>
+      </c>
+      <c r="P23">
+        <v>7</v>
+      </c>
+      <c r="Q23">
+        <v>92</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>1</v>
+      </c>
+      <c r="U23">
+        <v>6</v>
+      </c>
+      <c r="V23">
+        <v>10</v>
+      </c>
+      <c r="W23">
+        <v>1</v>
+      </c>
+      <c r="X23">
+        <v>1</v>
+      </c>
+      <c r="Y23">
+        <v>1</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>10</v>
+      </c>
+      <c r="AB23">
+        <v>30</v>
+      </c>
+      <c r="AC23">
+        <v>1</v>
+      </c>
+      <c r="AD23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>22/07/2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C24">
+        <v>1590</v>
+      </c>
+      <c r="D24">
+        <v>960</v>
+      </c>
+      <c r="E24">
+        <v>60</v>
+      </c>
+      <c r="F24">
+        <v>900</v>
+      </c>
+      <c r="G24">
+        <v>630</v>
+      </c>
+      <c r="H24">
+        <v>2</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>5</v>
+      </c>
+      <c r="K24">
+        <v>2</v>
+      </c>
+      <c r="L24">
+        <v>8</v>
+      </c>
+      <c r="M24">
+        <v>2</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>2</v>
+      </c>
+      <c r="P24">
+        <v>4</v>
+      </c>
+      <c r="Q24">
+        <v>25</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0.5</v>
+      </c>
+      <c r="U24">
+        <v>0.5</v>
+      </c>
+      <c r="V24">
+        <v>4</v>
+      </c>
+      <c r="W24">
+        <v>0.5</v>
+      </c>
+      <c r="X24">
+        <v>0.5</v>
+      </c>
+      <c r="Y24">
+        <v>0.5</v>
+      </c>
+      <c r="Z24">
+        <v>0.5</v>
+      </c>
+      <c r="AA24">
+        <v>4</v>
+      </c>
+      <c r="AB24">
+        <v>5</v>
+      </c>
+      <c r="AC24">
+        <v>2</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>23/07/2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C25">
+        <v>3110</v>
+      </c>
+      <c r="D25">
+        <v>1930</v>
+      </c>
+      <c r="E25">
+        <v>60</v>
+      </c>
+      <c r="F25">
+        <v>1870</v>
+      </c>
+      <c r="G25">
+        <v>1180</v>
+      </c>
+      <c r="H25">
+        <v>5</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>27</v>
+      </c>
+      <c r="K25">
+        <v>3</v>
+      </c>
+      <c r="L25">
+        <v>8</v>
+      </c>
+      <c r="M25">
+        <v>4</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>5</v>
+      </c>
+      <c r="P25">
+        <v>2</v>
+      </c>
+      <c r="Q25">
+        <v>54</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0.5</v>
+      </c>
+      <c r="U25">
+        <v>3</v>
+      </c>
+      <c r="V25">
+        <v>4</v>
+      </c>
+      <c r="W25">
+        <v>0.5</v>
+      </c>
+      <c r="X25">
+        <v>0.5</v>
+      </c>
+      <c r="Y25">
+        <v>0.5</v>
+      </c>
+      <c r="Z25">
+        <v>0.5</v>
+      </c>
+      <c r="AA25">
+        <v>6</v>
+      </c>
+      <c r="AB25">
+        <v>10</v>
+      </c>
+      <c r="AC25">
+        <v>1</v>
+      </c>
+      <c r="AD25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>24/07/2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C26">
+        <v>5530</v>
+      </c>
+      <c r="D26">
+        <v>3780</v>
+      </c>
+      <c r="E26">
+        <v>90</v>
+      </c>
+      <c r="F26">
+        <v>3690</v>
+      </c>
+      <c r="G26">
+        <v>1750</v>
+      </c>
+      <c r="H26">
+        <v>7</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>27</v>
+      </c>
+      <c r="K26">
+        <v>6</v>
+      </c>
+      <c r="L26">
+        <v>27</v>
+      </c>
+      <c r="M26">
+        <v>7</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>6</v>
+      </c>
+      <c r="P26">
+        <v>11</v>
+      </c>
+      <c r="Q26">
+        <v>91</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <v>0.5</v>
+      </c>
+      <c r="U26">
+        <v>3</v>
+      </c>
+      <c r="V26">
+        <v>12</v>
+      </c>
+      <c r="W26">
+        <v>2</v>
+      </c>
+      <c r="X26">
+        <v>2</v>
+      </c>
+      <c r="Y26">
+        <v>1</v>
+      </c>
+      <c r="Z26">
+        <v>1</v>
+      </c>
+      <c r="AA26">
+        <v>14</v>
+      </c>
+      <c r="AB26">
+        <v>17</v>
+      </c>
+      <c r="AC26">
+        <v>6</v>
+      </c>
+      <c r="AD26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>25/07/2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C27">
+        <v>5060</v>
+      </c>
+      <c r="D27">
+        <v>3010</v>
+      </c>
+      <c r="E27">
+        <v>90</v>
+      </c>
+      <c r="F27">
+        <v>2920</v>
+      </c>
+      <c r="G27">
+        <v>2050</v>
+      </c>
+      <c r="H27">
+        <v>7</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>41</v>
+      </c>
+      <c r="K27">
+        <v>3</v>
+      </c>
+      <c r="L27">
+        <v>17</v>
+      </c>
+      <c r="M27">
+        <v>7</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>4</v>
+      </c>
+      <c r="P27">
+        <v>8</v>
+      </c>
+      <c r="Q27">
+        <v>87</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27">
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <v>0.5</v>
+      </c>
+      <c r="U27">
+        <v>5</v>
+      </c>
+      <c r="V27">
+        <v>6</v>
+      </c>
+      <c r="W27">
+        <v>1.5</v>
+      </c>
+      <c r="X27">
+        <v>1.5</v>
+      </c>
+      <c r="Y27">
+        <v>1</v>
+      </c>
+      <c r="Z27">
+        <v>1</v>
+      </c>
+      <c r="AA27">
+        <v>14</v>
+      </c>
+      <c r="AB27">
+        <v>12</v>
+      </c>
+      <c r="AC27">
+        <v>5</v>
+      </c>
+      <c r="AD27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>26/07/2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C28">
+        <v>7760</v>
+      </c>
+      <c r="D28">
+        <v>4280</v>
+      </c>
+      <c r="E28">
+        <v>60</v>
+      </c>
+      <c r="F28">
+        <v>4220</v>
+      </c>
+      <c r="G28">
+        <v>3480</v>
+      </c>
+      <c r="H28">
+        <v>17</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>48</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+      <c r="L28">
+        <v>19</v>
+      </c>
+      <c r="M28">
+        <v>8</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>19</v>
+      </c>
+      <c r="P28">
+        <v>12</v>
+      </c>
+      <c r="Q28">
+        <v>128</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28">
+        <v>1</v>
+      </c>
+      <c r="U28">
+        <v>6</v>
+      </c>
+      <c r="V28">
+        <v>10</v>
+      </c>
+      <c r="W28">
+        <v>1.5</v>
+      </c>
+      <c r="X28">
+        <v>1.5</v>
+      </c>
+      <c r="Y28">
+        <v>1</v>
+      </c>
+      <c r="Z28">
+        <v>1</v>
+      </c>
+      <c r="AA28">
+        <v>16</v>
+      </c>
+      <c r="AB28">
+        <v>50</v>
+      </c>
+      <c r="AC28">
+        <v>8</v>
+      </c>
+      <c r="AD28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>27/07/2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C29">
+        <v>5040</v>
+      </c>
+      <c r="D29">
+        <v>3540</v>
+      </c>
+      <c r="E29">
+        <v>90</v>
+      </c>
+      <c r="F29">
+        <v>3450</v>
+      </c>
+      <c r="G29">
+        <v>1500</v>
+      </c>
+      <c r="H29">
+        <v>9</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>18</v>
+      </c>
+      <c r="K29">
+        <v>6</v>
+      </c>
+      <c r="L29">
+        <v>30</v>
+      </c>
+      <c r="M29">
+        <v>7</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>7</v>
+      </c>
+      <c r="P29">
+        <v>4</v>
+      </c>
+      <c r="Q29">
+        <v>81</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>0.5</v>
+      </c>
+      <c r="U29">
+        <v>3</v>
+      </c>
+      <c r="V29">
+        <v>12</v>
+      </c>
+      <c r="W29">
+        <v>2</v>
+      </c>
+      <c r="X29">
+        <v>2</v>
+      </c>
+      <c r="Y29">
+        <v>1</v>
+      </c>
+      <c r="Z29">
+        <v>1</v>
+      </c>
+      <c r="AA29">
+        <v>14</v>
+      </c>
+      <c r="AB29">
+        <v>14</v>
+      </c>
+      <c r="AC29">
+        <v>2</v>
+      </c>
+      <c r="AD29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C30">
+        <v>5750</v>
+      </c>
+      <c r="D30">
+        <v>3550</v>
+      </c>
+      <c r="E30">
+        <v>90</v>
+      </c>
+      <c r="F30">
+        <v>3460</v>
+      </c>
+      <c r="G30">
+        <v>2200</v>
+      </c>
+      <c r="H30">
+        <v>16</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>32</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+      <c r="L30">
+        <v>16</v>
+      </c>
+      <c r="M30">
+        <v>12</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>11</v>
+      </c>
+      <c r="P30">
+        <v>7</v>
+      </c>
+      <c r="Q30">
+        <v>97</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>1</v>
+      </c>
+      <c r="U30">
+        <v>5</v>
+      </c>
+      <c r="V30">
+        <v>5</v>
+      </c>
+      <c r="W30">
+        <v>1</v>
+      </c>
+      <c r="X30">
+        <v>1</v>
+      </c>
+      <c r="Y30">
+        <v>1</v>
+      </c>
+      <c r="Z30">
+        <v>1</v>
+      </c>
+      <c r="AA30">
+        <v>20</v>
+      </c>
+      <c r="AB30">
+        <v>21</v>
+      </c>
+      <c r="AC30">
+        <v>4</v>
+      </c>
+      <c r="AD30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>29/07/2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C31">
+        <v>3590</v>
+      </c>
+      <c r="D31">
+        <v>2730</v>
+      </c>
+      <c r="E31">
+        <v>60</v>
+      </c>
+      <c r="F31">
+        <v>2670</v>
+      </c>
+      <c r="G31">
+        <v>860</v>
+      </c>
+      <c r="H31">
+        <v>6</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>28</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+      <c r="L31">
+        <v>5</v>
+      </c>
+      <c r="M31">
+        <v>8</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>3</v>
+      </c>
+      <c r="P31">
+        <v>5</v>
+      </c>
+      <c r="Q31">
+        <v>60</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>0.5</v>
+      </c>
+      <c r="U31">
+        <v>4</v>
+      </c>
+      <c r="V31">
+        <v>10</v>
+      </c>
+      <c r="W31">
+        <v>0.5</v>
+      </c>
+      <c r="X31">
+        <v>0.5</v>
+      </c>
+      <c r="Y31">
+        <v>0.5</v>
+      </c>
+      <c r="Z31">
+        <v>0.5</v>
+      </c>
+      <c r="AA31">
+        <v>16</v>
+      </c>
+      <c r="AB31">
+        <v>6</v>
+      </c>
+      <c r="AC31">
+        <v>3</v>
+      </c>
+      <c r="AD31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>30/07/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C32">
+        <v>2760</v>
+      </c>
+      <c r="D32">
+        <v>1360</v>
+      </c>
+      <c r="E32">
+        <v>60</v>
+      </c>
+      <c r="F32">
+        <v>1300</v>
+      </c>
+      <c r="G32">
+        <v>1400</v>
+      </c>
+      <c r="H32">
+        <v>5</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>17</v>
+      </c>
+      <c r="K32">
+        <v>2</v>
+      </c>
+      <c r="L32">
+        <v>10</v>
+      </c>
+      <c r="M32">
+        <v>5</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>1</v>
+      </c>
+      <c r="P32">
+        <v>6</v>
+      </c>
+      <c r="Q32">
+        <v>46</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>0.5</v>
+      </c>
+      <c r="U32">
+        <v>2</v>
+      </c>
+      <c r="V32">
+        <v>4</v>
+      </c>
+      <c r="W32">
+        <v>2</v>
+      </c>
+      <c r="X32">
+        <v>0.5</v>
+      </c>
+      <c r="Y32">
+        <v>2</v>
+      </c>
+      <c r="Z32">
+        <v>2</v>
+      </c>
+      <c r="AA32">
+        <v>10</v>
+      </c>
+      <c r="AB32">
+        <v>2</v>
+      </c>
+      <c r="AC32">
+        <v>3</v>
+      </c>
+      <c r="AD32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C33">
+        <v>3020</v>
+      </c>
+      <c r="D33">
+        <v>2110</v>
+      </c>
+      <c r="E33">
+        <v>60</v>
+      </c>
+      <c r="F33">
+        <v>2050</v>
+      </c>
+      <c r="G33">
+        <v>910</v>
+      </c>
+      <c r="H33">
+        <v>5</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>24</v>
+      </c>
+      <c r="K33">
+        <v>3</v>
+      </c>
+      <c r="L33">
+        <v>11</v>
+      </c>
+      <c r="M33">
+        <v>3</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>5</v>
+      </c>
+      <c r="P33">
+        <v>1</v>
+      </c>
+      <c r="Q33">
+        <v>52</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>0.5</v>
+      </c>
+      <c r="U33">
+        <v>3</v>
+      </c>
+      <c r="V33">
+        <v>6</v>
+      </c>
+      <c r="W33">
+        <v>0.5</v>
+      </c>
+      <c r="X33">
+        <v>0.5</v>
+      </c>
+      <c r="Y33">
+        <v>0.5</v>
+      </c>
+      <c r="Z33">
+        <v>0.5</v>
+      </c>
+      <c r="AA33">
+        <v>6</v>
+      </c>
+      <c r="AB33">
+        <v>10</v>
+      </c>
+      <c r="AC33">
+        <v>1</v>
+      </c>
+      <c r="AD33">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>